<commit_message>
Forecast update 2026-07-26 (100 days out)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Data as of 2026-07-25 · evaluated at 0 days to election (actual: 101 days out)</t>
+          <t>Data as of 2026-07-26 · evaluated at 0 days to election (actual: 100 days out)</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>50.9</v>
+        <v>50</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,10 +566,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.1</v>
+        <v>231.9</v>
       </c>
       <c r="C9" t="n">
-        <v>202.9</v>
+        <v>203.1</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.3</v>
+        <v>24.5</v>
       </c>
       <c r="C10" t="n">
-        <v>25.7</v>
+        <v>25.5</v>
       </c>
       <c r="D10" t="n">
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>39.5</v>
+        <v>41.6</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.6</v>
+        <v>-2.86</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>39.1</v>
+        <v>41</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>60.9</v>
+        <v>59</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="AB2" s="4" t="n">
-        <v>44.4</v>
+        <v>44.38</v>
       </c>
       <c r="AC2" s="4" t="n">
-        <v>47.6</v>
+        <v>47.62</v>
       </c>
       <c r="AD2" s="4" t="n">
         <v>8</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>26.78</v>
+        <v>26.81</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>100</v>
@@ -1394,10 +1394,10 @@
         <v>0</v>
       </c>
       <c r="AB6" s="4" t="n">
-        <v>63.39</v>
+        <v>63.4</v>
       </c>
       <c r="AC6" s="4" t="n">
-        <v>36.61</v>
+        <v>36.6</v>
       </c>
       <c r="AD6" s="4" t="n">
         <v>0</v>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>17.56</v>
+        <v>17.6</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>99.59999999999999</v>
@@ -1610,10 +1610,10 @@
         <v>0</v>
       </c>
       <c r="AB8" s="4" t="n">
-        <v>58.78</v>
+        <v>58.8</v>
       </c>
       <c r="AC8" s="4" t="n">
-        <v>41.22</v>
+        <v>41.2</v>
       </c>
       <c r="AD8" s="4" t="n">
         <v>0</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>-6.05</v>
+        <v>-6.06</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>15.5</v>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2.88</v>
+        <v>2.86</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>73</v>
@@ -1818,10 +1818,10 @@
         <v>0</v>
       </c>
       <c r="AB10" s="4" t="n">
-        <v>51.44</v>
+        <v>51.43</v>
       </c>
       <c r="AC10" s="4" t="n">
-        <v>48.56</v>
+        <v>48.57</v>
       </c>
       <c r="AD10" s="4" t="n">
         <v>0</v>
@@ -2024,10 +2024,10 @@
         <v>0</v>
       </c>
       <c r="AB12" s="4" t="n">
-        <v>52.82</v>
+        <v>52.83</v>
       </c>
       <c r="AC12" s="4" t="n">
-        <v>47.18</v>
+        <v>47.17</v>
       </c>
       <c r="AD12" s="4" t="n">
         <v>0</v>
@@ -2383,7 +2383,7 @@
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>29.24</v>
+        <v>29.26</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>100</v>
@@ -2440,10 +2440,10 @@
         <v>0</v>
       </c>
       <c r="AB16" s="4" t="n">
-        <v>64.62</v>
+        <v>64.63</v>
       </c>
       <c r="AC16" s="4" t="n">
-        <v>35.38</v>
+        <v>35.37</v>
       </c>
       <c r="AD16" s="4" t="n">
         <v>0</v>
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="I18" s="4" t="n">
-        <v>12.58</v>
+        <v>12.56</v>
       </c>
       <c r="J18" s="4" t="n">
         <v>99</v>
@@ -2656,10 +2656,10 @@
         <v>0</v>
       </c>
       <c r="AB18" s="4" t="n">
-        <v>55.65</v>
+        <v>55.64</v>
       </c>
       <c r="AC18" s="4" t="n">
-        <v>43.21</v>
+        <v>43.22</v>
       </c>
       <c r="AD18" s="4" t="n">
         <v>0</v>
@@ -2703,7 +2703,7 @@
         </is>
       </c>
       <c r="I19" s="4" t="n">
-        <v>12.39</v>
+        <v>12.4</v>
       </c>
       <c r="J19" s="4" t="n">
         <v>98.90000000000001</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>12.48</v>
+        <v>12.47</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>98.90000000000001</v>
@@ -2864,10 +2864,10 @@
         <v>0</v>
       </c>
       <c r="AB20" s="4" t="n">
-        <v>56.24</v>
+        <v>56.23</v>
       </c>
       <c r="AC20" s="4" t="n">
-        <v>43.76</v>
+        <v>43.77</v>
       </c>
       <c r="AD20" s="4" t="n">
         <v>0</v>
@@ -3027,13 +3027,13 @@
         </is>
       </c>
       <c r="I22" s="4" t="n">
-        <v>-10.6</v>
+        <v>-10.61</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>97.2</v>
+        <v>97.3</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -3084,10 +3084,10 @@
         <v>0</v>
       </c>
       <c r="AB22" s="4" t="n">
-        <v>44.7</v>
+        <v>44.69</v>
       </c>
       <c r="AC22" s="4" t="n">
-        <v>55.3</v>
+        <v>55.31</v>
       </c>
       <c r="AD22" s="4" t="n">
         <v>0</v>
@@ -3131,13 +3131,13 @@
         </is>
       </c>
       <c r="I23" s="4" t="n">
-        <v>6.63</v>
+        <v>6.68</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>86.3</v>
+        <v>86.5</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -3188,10 +3188,10 @@
         <v>0</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>53.31</v>
+        <v>53.34</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>46.69</v>
+        <v>46.66</v>
       </c>
       <c r="AD23" s="4" t="n">
         <v>0</v>
@@ -3239,7 +3239,7 @@
         </is>
       </c>
       <c r="I24" s="4" t="n">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
       <c r="J24" s="4" t="n">
         <v>67.8</v>
@@ -3296,10 +3296,10 @@
         <v>0</v>
       </c>
       <c r="AB24" s="4" t="n">
-        <v>50.76</v>
+        <v>50.77</v>
       </c>
       <c r="AC24" s="4" t="n">
-        <v>49.24</v>
+        <v>49.23</v>
       </c>
       <c r="AD24" s="4" t="n">
         <v>0</v>
@@ -3347,7 +3347,7 @@
         </is>
       </c>
       <c r="I25" s="4" t="n">
-        <v>15.13</v>
+        <v>15.12</v>
       </c>
       <c r="J25" s="4" t="n">
         <v>99.3</v>
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="I26" s="4" t="n">
-        <v>-3.37</v>
+        <v>-3.38</v>
       </c>
       <c r="J26" s="4" t="n">
         <v>25.1</v>
@@ -3508,10 +3508,10 @@
         <v>0</v>
       </c>
       <c r="AB26" s="4" t="n">
-        <v>48.32</v>
+        <v>48.31</v>
       </c>
       <c r="AC26" s="4" t="n">
-        <v>51.68</v>
+        <v>51.69</v>
       </c>
       <c r="AD26" s="4" t="n">
         <v>0</v>
@@ -3657,13 +3657,13 @@
         </is>
       </c>
       <c r="I28" s="4" t="n">
-        <v>4.37</v>
+        <v>4.39</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>78.59999999999999</v>
+        <v>78.7</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="I29" s="4" t="n">
-        <v>16.45</v>
+        <v>16.46</v>
       </c>
       <c r="J29" s="4" t="n">
         <v>99.5</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>19.57</v>
+        <v>19.59</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>99.7</v>
@@ -4226,10 +4226,10 @@
         <v>0</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>39.42</v>
+        <v>39.43</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>60.58</v>
+        <v>60.57</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>0</v>
@@ -4277,7 +4277,7 @@
         </is>
       </c>
       <c r="I34" s="4" t="n">
-        <v>-8.6</v>
+        <v>-8.609999999999999</v>
       </c>
       <c r="J34" s="4" t="n">
         <v>7.8</v>
@@ -4385,7 +4385,7 @@
         </is>
       </c>
       <c r="I35" s="4" t="n">
-        <v>-18.56</v>
+        <v>-18.66</v>
       </c>
       <c r="J35" s="4" t="n">
         <v>0.3</v>
@@ -4442,10 +4442,10 @@
         <v>0</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>40.72</v>
+        <v>40.67</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>59.28</v>
+        <v>59.33</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>0</v>
@@ -4489,13 +4489,13 @@
         </is>
       </c>
       <c r="I36" s="4" t="n">
-        <v>1.9</v>
+        <v>1.92</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>69.2</v>
+        <v>69.3</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>30.8</v>
+        <v>30.7</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -4546,10 +4546,10 @@
         <v>0</v>
       </c>
       <c r="AB36" s="4" t="n">
-        <v>50.95</v>
+        <v>50.96</v>
       </c>
       <c r="AC36" s="4" t="n">
-        <v>49.05</v>
+        <v>49.04</v>
       </c>
       <c r="AD36" s="4" t="n">
         <v>0</v>
@@ -4695,27 +4695,27 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-3.19</v>
+        <v>-2.96</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>38.9</v>
+        <v>41.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>61.1</v>
+        <v>58.9</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.71</v>
+        <v>-2.51</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.41</v>
+        <v>-1.21</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.1</v>
@@ -4750,16 +4750,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.41</v>
+        <v>48.52</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>38.9</v>
+        <v>41.1</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.59</v>
+        <v>51.48</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -4962,10 +4962,10 @@
         <v>0</v>
       </c>
       <c r="AB40" s="4" t="n">
-        <v>48.4</v>
+        <v>48.41</v>
       </c>
       <c r="AC40" s="4" t="n">
-        <v>51.6</v>
+        <v>51.59</v>
       </c>
       <c r="AD40" s="4" t="n">
         <v>0</v>
@@ -6035,13 +6035,13 @@
         </is>
       </c>
       <c r="I51" s="4" t="n">
-        <v>-0.76</v>
+        <v>-0.72</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>64.7</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -6092,10 +6092,10 @@
         <v>0</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>49.62</v>
+        <v>49.64</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>50.38</v>
+        <v>50.36</v>
       </c>
       <c r="AD51" s="4" t="n">
         <v>0</v>
@@ -6445,7 +6445,7 @@
         </is>
       </c>
       <c r="I55" s="4" t="n">
-        <v>4.79</v>
+        <v>4.8</v>
       </c>
       <c r="J55" s="4" t="n">
         <v>80.09999999999999</v>
@@ -6502,10 +6502,10 @@
         <v>0</v>
       </c>
       <c r="AB55" s="4" t="n">
-        <v>51.28</v>
+        <v>51.29</v>
       </c>
       <c r="AC55" s="4" t="n">
-        <v>46.6</v>
+        <v>46.59</v>
       </c>
       <c r="AD55" s="4" t="n">
         <v>2.12</v>
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="M59" s="4" t="n">
-        <v>15.45</v>
+        <v>15.46</v>
       </c>
       <c r="N59" s="4" t="n">
         <v>5.13</v>
@@ -6961,7 +6961,7 @@
         </is>
       </c>
       <c r="I60" s="4" t="n">
-        <v>33.31</v>
+        <v>33.32</v>
       </c>
       <c r="J60" s="4" t="n">
         <v>100</v>
@@ -6975,13 +6975,13 @@
         </is>
       </c>
       <c r="M60" s="4" t="n">
-        <v>27.83</v>
+        <v>27.84</v>
       </c>
       <c r="N60" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O60" s="4" t="n">
-        <v>33.31</v>
+        <v>33.32</v>
       </c>
       <c r="P60" s="4" t="n">
         <v>0</v>
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="I61" s="4" t="n">
-        <v>21.12</v>
+        <v>21.13</v>
       </c>
       <c r="J61" s="4" t="n">
         <v>99.8</v>
@@ -7083,7 +7083,7 @@
         <v>5.13</v>
       </c>
       <c r="O61" s="4" t="n">
-        <v>21.12</v>
+        <v>21.13</v>
       </c>
       <c r="P61" s="4" t="n">
         <v>1.08</v>
@@ -7179,13 +7179,13 @@
         </is>
       </c>
       <c r="M62" s="4" t="n">
-        <v>18.28</v>
+        <v>18.29</v>
       </c>
       <c r="N62" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O62" s="4" t="n">
-        <v>26.54</v>
+        <v>26.55</v>
       </c>
       <c r="P62" s="4" t="n">
         <v>0</v>
@@ -7267,7 +7267,7 @@
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>-18.24</v>
+        <v>-18.23</v>
       </c>
       <c r="J63" s="4" t="n">
         <v>0.3</v>
@@ -7287,7 +7287,7 @@
         <v>5.13</v>
       </c>
       <c r="O63" s="4" t="n">
-        <v>-18.24</v>
+        <v>-18.23</v>
       </c>
       <c r="P63" s="4" t="n">
         <v>-0.65</v>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="I64" s="4" t="n">
-        <v>12.39</v>
+        <v>12.4</v>
       </c>
       <c r="J64" s="4" t="n">
         <v>98.90000000000001</v>
@@ -7383,13 +7383,13 @@
         </is>
       </c>
       <c r="M64" s="4" t="n">
-        <v>11.25</v>
+        <v>11.26</v>
       </c>
       <c r="N64" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>12.39</v>
+        <v>12.4</v>
       </c>
       <c r="P64" s="4" t="n">
         <v>-0.35</v>
@@ -7491,7 +7491,7 @@
         <v>5.13</v>
       </c>
       <c r="O65" s="4" t="n">
-        <v>25.41</v>
+        <v>25.42</v>
       </c>
       <c r="P65" s="4" t="n">
         <v>0</v>
@@ -7587,7 +7587,7 @@
         </is>
       </c>
       <c r="M66" s="4" t="n">
-        <v>39.18</v>
+        <v>39.19</v>
       </c>
       <c r="N66" s="4" t="n">
         <v>5.13</v>
@@ -7624,10 +7624,10 @@
         <v>0</v>
       </c>
       <c r="AB66" s="4" t="n">
-        <v>74.48</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="AC66" s="4" t="n">
-        <v>25.52</v>
+        <v>25.51</v>
       </c>
       <c r="AD66" s="4" t="n">
         <v>0</v>
@@ -7675,7 +7675,7 @@
         </is>
       </c>
       <c r="I67" s="4" t="n">
-        <v>30.7</v>
+        <v>30.71</v>
       </c>
       <c r="J67" s="4" t="n">
         <v>100</v>
@@ -7695,7 +7695,7 @@
         <v>5.13</v>
       </c>
       <c r="O67" s="4" t="n">
-        <v>30.7</v>
+        <v>30.71</v>
       </c>
       <c r="P67" s="4" t="n">
         <v>2.78</v>
@@ -7777,7 +7777,7 @@
         </is>
       </c>
       <c r="I68" s="4" t="n">
-        <v>42.87</v>
+        <v>42.88</v>
       </c>
       <c r="J68" s="4" t="n">
         <v>100</v>
@@ -7797,7 +7797,7 @@
         <v>5.13</v>
       </c>
       <c r="O68" s="4" t="n">
-        <v>42.87</v>
+        <v>42.88</v>
       </c>
       <c r="P68" s="4" t="n">
         <v>0</v>
@@ -7889,13 +7889,13 @@
         </is>
       </c>
       <c r="M69" s="4" t="n">
-        <v>74.04000000000001</v>
+        <v>74.05</v>
       </c>
       <c r="N69" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O69" s="4" t="n">
-        <v>78.86</v>
+        <v>78.87</v>
       </c>
       <c r="P69" s="4" t="n">
         <v>0</v>
@@ -8079,7 +8079,7 @@
         </is>
       </c>
       <c r="I71" s="4" t="n">
-        <v>21.59</v>
+        <v>21.6</v>
       </c>
       <c r="J71" s="4" t="n">
         <v>99.8</v>
@@ -8099,7 +8099,7 @@
         <v>5.13</v>
       </c>
       <c r="O71" s="4" t="n">
-        <v>21.59</v>
+        <v>21.6</v>
       </c>
       <c r="P71" s="4" t="n">
         <v>0.46</v>
@@ -8191,13 +8191,13 @@
         </is>
       </c>
       <c r="M72" s="4" t="n">
-        <v>40.71</v>
+        <v>40.72</v>
       </c>
       <c r="N72" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>45.96</v>
+        <v>45.97</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
@@ -8330,10 +8330,10 @@
         <v>0</v>
       </c>
       <c r="AB73" s="4" t="n">
-        <v>79.09999999999999</v>
+        <v>79.11</v>
       </c>
       <c r="AC73" s="4" t="n">
-        <v>20.9</v>
+        <v>20.89</v>
       </c>
       <c r="AD73" s="4" t="n">
         <v>0</v>
@@ -8395,7 +8395,7 @@
         </is>
       </c>
       <c r="M74" s="4" t="n">
-        <v>52.92</v>
+        <v>52.93</v>
       </c>
       <c r="N74" s="4" t="n">
         <v>5.13</v>
@@ -8483,7 +8483,7 @@
         </is>
       </c>
       <c r="I75" s="4" t="n">
-        <v>48.97</v>
+        <v>48.98</v>
       </c>
       <c r="J75" s="4" t="n">
         <v>100</v>
@@ -8503,7 +8503,7 @@
         <v>5.13</v>
       </c>
       <c r="O75" s="4" t="n">
-        <v>48.97</v>
+        <v>48.98</v>
       </c>
       <c r="P75" s="4" t="n">
         <v>3.69</v>
@@ -8585,7 +8585,7 @@
         </is>
       </c>
       <c r="I76" s="4" t="n">
-        <v>43.91</v>
+        <v>43.92</v>
       </c>
       <c r="J76" s="4" t="n">
         <v>100</v>
@@ -8605,7 +8605,7 @@
         <v>5.13</v>
       </c>
       <c r="O76" s="4" t="n">
-        <v>43.91</v>
+        <v>43.92</v>
       </c>
       <c r="P76" s="4" t="n">
         <v>2.1</v>
@@ -8701,13 +8701,13 @@
         </is>
       </c>
       <c r="M77" s="4" t="n">
-        <v>38.65</v>
+        <v>38.66</v>
       </c>
       <c r="N77" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O77" s="4" t="n">
-        <v>50.18</v>
+        <v>50.19</v>
       </c>
       <c r="P77" s="4" t="n">
         <v>2.46</v>
@@ -8789,7 +8789,7 @@
         </is>
       </c>
       <c r="I78" s="4" t="n">
-        <v>-28.63</v>
+        <v>-28.62</v>
       </c>
       <c r="J78" s="4" t="n">
         <v>0</v>
@@ -8803,13 +8803,13 @@
         </is>
       </c>
       <c r="M78" s="4" t="n">
-        <v>-30.32</v>
+        <v>-30.31</v>
       </c>
       <c r="N78" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O78" s="4" t="n">
-        <v>-28.63</v>
+        <v>-28.62</v>
       </c>
       <c r="P78" s="4" t="n">
         <v>-2.51</v>
@@ -8905,7 +8905,7 @@
         </is>
       </c>
       <c r="M79" s="4" t="n">
-        <v>11.79</v>
+        <v>11.8</v>
       </c>
       <c r="N79" s="4" t="n">
         <v>5.13</v>
@@ -8993,13 +8993,13 @@
         </is>
       </c>
       <c r="I80" s="4" t="n">
-        <v>5.43</v>
+        <v>5.45</v>
       </c>
       <c r="J80" s="4" t="n">
-        <v>82.3</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -9007,7 +9007,7 @@
         </is>
       </c>
       <c r="M80" s="4" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="N80" s="4" t="n">
         <v>5.13</v>
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="AB80" s="4" t="n">
-        <v>52.71</v>
+        <v>52.72</v>
       </c>
       <c r="AC80" s="4" t="n">
-        <v>47.29</v>
+        <v>47.28</v>
       </c>
       <c r="AD80" s="4" t="n">
         <v>0</v>
@@ -9217,7 +9217,7 @@
         </is>
       </c>
       <c r="M82" s="4" t="n">
-        <v>28.2</v>
+        <v>28.21</v>
       </c>
       <c r="N82" s="4" t="n">
         <v>5.13</v>
@@ -9254,10 +9254,10 @@
         <v>0</v>
       </c>
       <c r="AB82" s="4" t="n">
-        <v>68.31</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="AC82" s="4" t="n">
-        <v>31.69</v>
+        <v>31.68</v>
       </c>
       <c r="AD82" s="4" t="n">
         <v>0</v>
@@ -9356,10 +9356,10 @@
         <v>0</v>
       </c>
       <c r="AB83" s="4" t="n">
-        <v>59.86</v>
+        <v>59.87</v>
       </c>
       <c r="AC83" s="4" t="n">
-        <v>40.14</v>
+        <v>40.13</v>
       </c>
       <c r="AD83" s="4" t="n">
         <v>0</v>
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="I84" s="4" t="n">
-        <v>25.79</v>
+        <v>25.8</v>
       </c>
       <c r="J84" s="4" t="n">
         <v>100</v>
@@ -9423,7 +9423,7 @@
         <v>5.13</v>
       </c>
       <c r="O84" s="4" t="n">
-        <v>25.79</v>
+        <v>25.8</v>
       </c>
       <c r="P84" s="4" t="n">
         <v>0.63</v>
@@ -9607,7 +9607,7 @@
         </is>
       </c>
       <c r="I86" s="4" t="n">
-        <v>39.75</v>
+        <v>39.76</v>
       </c>
       <c r="J86" s="4" t="n">
         <v>100</v>
@@ -9621,13 +9621,13 @@
         </is>
       </c>
       <c r="M86" s="4" t="n">
-        <v>29.79</v>
+        <v>29.8</v>
       </c>
       <c r="N86" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O86" s="4" t="n">
-        <v>39.75</v>
+        <v>39.76</v>
       </c>
       <c r="P86" s="4" t="n">
         <v>2.23</v>
@@ -9723,7 +9723,7 @@
         </is>
       </c>
       <c r="M87" s="4" t="n">
-        <v>41.35</v>
+        <v>41.36</v>
       </c>
       <c r="N87" s="4" t="n">
         <v>5.13</v>
@@ -9811,7 +9811,7 @@
         </is>
       </c>
       <c r="I88" s="4" t="n">
-        <v>51.65</v>
+        <v>51.66</v>
       </c>
       <c r="J88" s="4" t="n">
         <v>100</v>
@@ -9825,13 +9825,13 @@
         </is>
       </c>
       <c r="M88" s="4" t="n">
-        <v>44.8</v>
+        <v>44.81</v>
       </c>
       <c r="N88" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O88" s="4" t="n">
-        <v>51.65</v>
+        <v>51.66</v>
       </c>
       <c r="P88" s="4" t="n">
         <v>1.57</v>
@@ -9964,10 +9964,10 @@
         <v>0</v>
       </c>
       <c r="AB89" s="4" t="n">
-        <v>58.01</v>
+        <v>58.02</v>
       </c>
       <c r="AC89" s="4" t="n">
-        <v>41.99</v>
+        <v>41.98</v>
       </c>
       <c r="AD89" s="4" t="n">
         <v>0</v>
@@ -10029,7 +10029,7 @@
         </is>
       </c>
       <c r="M90" s="4" t="n">
-        <v>29.91</v>
+        <v>29.92</v>
       </c>
       <c r="N90" s="4" t="n">
         <v>5.13</v>
@@ -10066,10 +10066,10 @@
         <v>0</v>
       </c>
       <c r="AB90" s="4" t="n">
-        <v>69.75</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="AC90" s="4" t="n">
-        <v>30.25</v>
+        <v>30.24</v>
       </c>
       <c r="AD90" s="4" t="n">
         <v>0</v>
@@ -10117,7 +10117,7 @@
         </is>
       </c>
       <c r="I91" s="4" t="n">
-        <v>28.34</v>
+        <v>28.35</v>
       </c>
       <c r="J91" s="4" t="n">
         <v>100</v>
@@ -10131,13 +10131,13 @@
         </is>
       </c>
       <c r="M91" s="4" t="n">
-        <v>16.26</v>
+        <v>16.27</v>
       </c>
       <c r="N91" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O91" s="4" t="n">
-        <v>28.34</v>
+        <v>28.35</v>
       </c>
       <c r="P91" s="4" t="n">
         <v>0</v>
@@ -10233,7 +10233,7 @@
         </is>
       </c>
       <c r="M92" s="4" t="n">
-        <v>58.82</v>
+        <v>58.83</v>
       </c>
       <c r="N92" s="4" t="n">
         <v>5.13</v>
@@ -10321,7 +10321,7 @@
         </is>
       </c>
       <c r="I93" s="4" t="n">
-        <v>26.25</v>
+        <v>26.26</v>
       </c>
       <c r="J93" s="4" t="n">
         <v>100</v>
@@ -10341,7 +10341,7 @@
         <v>5.13</v>
       </c>
       <c r="O93" s="4" t="n">
-        <v>26.25</v>
+        <v>26.26</v>
       </c>
       <c r="P93" s="4" t="n">
         <v>2.03</v>
@@ -10423,7 +10423,7 @@
         </is>
       </c>
       <c r="I94" s="4" t="n">
-        <v>51.03</v>
+        <v>51.04</v>
       </c>
       <c r="J94" s="4" t="n">
         <v>100</v>
@@ -10437,13 +10437,13 @@
         </is>
       </c>
       <c r="M94" s="4" t="n">
-        <v>43.41</v>
+        <v>43.42</v>
       </c>
       <c r="N94" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O94" s="4" t="n">
-        <v>51.03</v>
+        <v>51.04</v>
       </c>
       <c r="P94" s="4" t="n">
         <v>2.66</v>
@@ -10545,7 +10545,7 @@
         <v>5.13</v>
       </c>
       <c r="O95" s="4" t="n">
-        <v>76.52</v>
+        <v>76.53</v>
       </c>
       <c r="P95" s="4" t="n">
         <v>0</v>
@@ -10674,10 +10674,10 @@
         <v>0</v>
       </c>
       <c r="AB96" s="4" t="n">
-        <v>62.98</v>
+        <v>62.99</v>
       </c>
       <c r="AC96" s="4" t="n">
-        <v>37.02</v>
+        <v>37.01</v>
       </c>
       <c r="AD96" s="4" t="n">
         <v>0</v>
@@ -10929,7 +10929,7 @@
         </is>
       </c>
       <c r="I99" s="4" t="n">
-        <v>31.1</v>
+        <v>31.11</v>
       </c>
       <c r="J99" s="4" t="n">
         <v>100</v>
@@ -10949,7 +10949,7 @@
         <v>5.13</v>
       </c>
       <c r="O99" s="4" t="n">
-        <v>31.1</v>
+        <v>31.11</v>
       </c>
       <c r="P99" s="4" t="n">
         <v>2.64</v>
@@ -11031,7 +11031,7 @@
         </is>
       </c>
       <c r="I100" s="4" t="n">
-        <v>26.2</v>
+        <v>26.21</v>
       </c>
       <c r="J100" s="4" t="n">
         <v>100</v>
@@ -11051,7 +11051,7 @@
         <v>5.13</v>
       </c>
       <c r="O100" s="4" t="n">
-        <v>26.2</v>
+        <v>26.21</v>
       </c>
       <c r="P100" s="4" t="n">
         <v>1.69</v>
@@ -11235,7 +11235,7 @@
         </is>
       </c>
       <c r="I102" s="4" t="n">
-        <v>58.85</v>
+        <v>58.86</v>
       </c>
       <c r="J102" s="4" t="n">
         <v>100</v>
@@ -11249,13 +11249,13 @@
         </is>
       </c>
       <c r="M102" s="4" t="n">
-        <v>43.5</v>
+        <v>43.51</v>
       </c>
       <c r="N102" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O102" s="4" t="n">
-        <v>58.85</v>
+        <v>58.86</v>
       </c>
       <c r="P102" s="4" t="n">
         <v>1.93</v>
@@ -11337,7 +11337,7 @@
         </is>
       </c>
       <c r="I103" s="4" t="n">
-        <v>20.23</v>
+        <v>20.24</v>
       </c>
       <c r="J103" s="4" t="n">
         <v>99.8</v>
@@ -11357,7 +11357,7 @@
         <v>5.13</v>
       </c>
       <c r="O103" s="4" t="n">
-        <v>20.23</v>
+        <v>20.24</v>
       </c>
       <c r="P103" s="4" t="n">
         <v>1.39</v>
@@ -11439,7 +11439,7 @@
         </is>
       </c>
       <c r="I104" s="4" t="n">
-        <v>39.35</v>
+        <v>39.36</v>
       </c>
       <c r="J104" s="4" t="n">
         <v>100</v>
@@ -11453,13 +11453,13 @@
         </is>
       </c>
       <c r="M104" s="4" t="n">
-        <v>21.96</v>
+        <v>21.97</v>
       </c>
       <c r="N104" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O104" s="4" t="n">
-        <v>39.35</v>
+        <v>39.36</v>
       </c>
       <c r="P104" s="4" t="n">
         <v>1.73</v>
@@ -11561,7 +11561,7 @@
         <v>5.13</v>
       </c>
       <c r="O105" s="4" t="n">
-        <v>22.44</v>
+        <v>22.45</v>
       </c>
       <c r="P105" s="4" t="n">
         <v>1.61</v>
@@ -11639,7 +11639,7 @@
         </is>
       </c>
       <c r="I106" s="4" t="n">
-        <v>11.7</v>
+        <v>11.71</v>
       </c>
       <c r="J106" s="4" t="n">
         <v>98.8</v>
@@ -11653,13 +11653,13 @@
         </is>
       </c>
       <c r="M106" s="4" t="n">
-        <v>5.58</v>
+        <v>5.59</v>
       </c>
       <c r="N106" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O106" s="4" t="n">
-        <v>11.7</v>
+        <v>11.71</v>
       </c>
       <c r="P106" s="4" t="n">
         <v>0.13</v>
@@ -11843,7 +11843,7 @@
         </is>
       </c>
       <c r="I108" s="4" t="n">
-        <v>26.17</v>
+        <v>26.18</v>
       </c>
       <c r="J108" s="4" t="n">
         <v>100</v>
@@ -11857,13 +11857,13 @@
         </is>
       </c>
       <c r="M108" s="4" t="n">
-        <v>20.74</v>
+        <v>20.75</v>
       </c>
       <c r="N108" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O108" s="4" t="n">
-        <v>26.17</v>
+        <v>26.18</v>
       </c>
       <c r="P108" s="4" t="n">
         <v>0</v>
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="I109" s="4" t="n">
-        <v>27.4</v>
+        <v>27.41</v>
       </c>
       <c r="J109" s="4" t="n">
         <v>100</v>
@@ -11959,13 +11959,13 @@
         </is>
       </c>
       <c r="M109" s="4" t="n">
-        <v>21.39</v>
+        <v>21.4</v>
       </c>
       <c r="N109" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O109" s="4" t="n">
-        <v>27.4</v>
+        <v>27.41</v>
       </c>
       <c r="P109" s="4" t="n">
         <v>0</v>
@@ -12047,7 +12047,7 @@
         </is>
       </c>
       <c r="I110" s="4" t="n">
-        <v>39.65</v>
+        <v>39.66</v>
       </c>
       <c r="J110" s="4" t="n">
         <v>100</v>
@@ -12067,7 +12067,7 @@
         <v>5.13</v>
       </c>
       <c r="O110" s="4" t="n">
-        <v>39.65</v>
+        <v>39.66</v>
       </c>
       <c r="P110" s="4" t="n">
         <v>1.58</v>
@@ -12973,7 +12973,7 @@
         </is>
       </c>
       <c r="I119" s="4" t="n">
-        <v>36.68</v>
+        <v>36.69</v>
       </c>
       <c r="J119" s="4" t="n">
         <v>100</v>
@@ -12987,13 +12987,13 @@
         </is>
       </c>
       <c r="M119" s="4" t="n">
-        <v>25.14</v>
+        <v>25.15</v>
       </c>
       <c r="N119" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O119" s="4" t="n">
-        <v>36.68</v>
+        <v>36.69</v>
       </c>
       <c r="P119" s="4" t="n">
         <v>2.93</v>
@@ -13075,7 +13075,7 @@
         </is>
       </c>
       <c r="I120" s="4" t="n">
-        <v>27.15</v>
+        <v>27.16</v>
       </c>
       <c r="J120" s="4" t="n">
         <v>100</v>
@@ -13089,13 +13089,13 @@
         </is>
       </c>
       <c r="M120" s="4" t="n">
-        <v>9.08</v>
+        <v>9.09</v>
       </c>
       <c r="N120" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O120" s="4" t="n">
-        <v>27.15</v>
+        <v>27.16</v>
       </c>
       <c r="P120" s="4" t="n">
         <v>1.43</v>
@@ -13177,7 +13177,7 @@
         </is>
       </c>
       <c r="I121" s="4" t="n">
-        <v>28.19</v>
+        <v>28.2</v>
       </c>
       <c r="J121" s="4" t="n">
         <v>100</v>
@@ -13191,13 +13191,13 @@
         </is>
       </c>
       <c r="M121" s="4" t="n">
-        <v>16.21</v>
+        <v>16.22</v>
       </c>
       <c r="N121" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O121" s="4" t="n">
-        <v>28.19</v>
+        <v>28.2</v>
       </c>
       <c r="P121" s="4" t="n">
         <v>2.19</v>
@@ -13279,7 +13279,7 @@
         </is>
       </c>
       <c r="I122" s="4" t="n">
-        <v>34.69</v>
+        <v>34.7</v>
       </c>
       <c r="J122" s="4" t="n">
         <v>100</v>
@@ -13293,13 +13293,13 @@
         </is>
       </c>
       <c r="M122" s="4" t="n">
-        <v>26.12</v>
+        <v>26.13</v>
       </c>
       <c r="N122" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O122" s="4" t="n">
-        <v>34.69</v>
+        <v>34.7</v>
       </c>
       <c r="P122" s="4" t="n">
         <v>2.06</v>
@@ -13381,7 +13381,7 @@
         </is>
       </c>
       <c r="I123" s="4" t="n">
-        <v>15.11</v>
+        <v>15.12</v>
       </c>
       <c r="J123" s="4" t="n">
         <v>99.3</v>
@@ -13395,13 +13395,13 @@
         </is>
       </c>
       <c r="M123" s="4" t="n">
-        <v>7.37</v>
+        <v>7.38</v>
       </c>
       <c r="N123" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O123" s="4" t="n">
-        <v>15.11</v>
+        <v>15.12</v>
       </c>
       <c r="P123" s="4" t="n">
         <v>1.9</v>
@@ -13432,10 +13432,10 @@
         <v>0</v>
       </c>
       <c r="AB123" s="4" t="n">
-        <v>57.55</v>
+        <v>57.56</v>
       </c>
       <c r="AC123" s="4" t="n">
-        <v>42.45</v>
+        <v>42.44</v>
       </c>
       <c r="AD123" s="4" t="n">
         <v>0</v>
@@ -14193,7 +14193,7 @@
         </is>
       </c>
       <c r="I131" s="4" t="n">
-        <v>-4.28</v>
+        <v>-4.29</v>
       </c>
       <c r="J131" s="4" t="n">
         <v>21.7</v>
@@ -16541,7 +16541,7 @@
         </is>
       </c>
       <c r="I154" s="4" t="n">
-        <v>24.24</v>
+        <v>24.23</v>
       </c>
       <c r="J154" s="4" t="n">
         <v>99.90000000000001</v>
@@ -16561,7 +16561,7 @@
         <v>5.13</v>
       </c>
       <c r="O154" s="4" t="n">
-        <v>24.24</v>
+        <v>24.23</v>
       </c>
       <c r="P154" s="4" t="n">
         <v>1.36</v>
@@ -16643,7 +16643,7 @@
         </is>
       </c>
       <c r="I155" s="4" t="n">
-        <v>-29.17</v>
+        <v>-29.18</v>
       </c>
       <c r="J155" s="4" t="n">
         <v>0</v>
@@ -16663,7 +16663,7 @@
         <v>5.13</v>
       </c>
       <c r="O155" s="4" t="n">
-        <v>-29.17</v>
+        <v>-29.18</v>
       </c>
       <c r="P155" s="4" t="n">
         <v>-1.75</v>
@@ -16847,7 +16847,7 @@
         </is>
       </c>
       <c r="I157" s="4" t="n">
-        <v>83.79000000000001</v>
+        <v>83.78</v>
       </c>
       <c r="J157" s="4" t="n">
         <v>100</v>
@@ -16867,7 +16867,7 @@
         <v>5.13</v>
       </c>
       <c r="O157" s="4" t="n">
-        <v>83.79000000000001</v>
+        <v>83.78</v>
       </c>
       <c r="P157" s="4" t="n">
         <v>0</v>
@@ -16949,7 +16949,7 @@
         </is>
       </c>
       <c r="I158" s="4" t="n">
-        <v>63.09</v>
+        <v>63.08</v>
       </c>
       <c r="J158" s="4" t="n">
         <v>100</v>
@@ -16969,7 +16969,7 @@
         <v>5.13</v>
       </c>
       <c r="O158" s="4" t="n">
-        <v>63.09</v>
+        <v>63.08</v>
       </c>
       <c r="P158" s="4" t="n">
         <v>2.07</v>
@@ -17553,7 +17553,7 @@
         </is>
       </c>
       <c r="I164" s="4" t="n">
-        <v>-11.69</v>
+        <v>-11.7</v>
       </c>
       <c r="J164" s="4" t="n">
         <v>1.2</v>
@@ -17573,7 +17573,7 @@
         <v>5.13</v>
       </c>
       <c r="O164" s="4" t="n">
-        <v>-11.69</v>
+        <v>-11.7</v>
       </c>
       <c r="P164" s="4" t="n">
         <v>-1.96</v>
@@ -17651,7 +17651,7 @@
         </is>
       </c>
       <c r="I165" s="4" t="n">
-        <v>50.88</v>
+        <v>50.87</v>
       </c>
       <c r="J165" s="4" t="n">
         <v>100</v>
@@ -17665,13 +17665,13 @@
         </is>
       </c>
       <c r="M165" s="4" t="n">
-        <v>45.48</v>
+        <v>45.47</v>
       </c>
       <c r="N165" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O165" s="4" t="n">
-        <v>50.88</v>
+        <v>50.87</v>
       </c>
       <c r="P165" s="4" t="n">
         <v>0</v>
@@ -18477,7 +18477,7 @@
         </is>
       </c>
       <c r="I173" s="4" t="n">
-        <v>-27.53</v>
+        <v>-27.84</v>
       </c>
       <c r="J173" s="4" t="n">
         <v>0</v>
@@ -18534,10 +18534,10 @@
         <v>0</v>
       </c>
       <c r="AB173" s="4" t="n">
-        <v>36.23</v>
+        <v>36.08</v>
       </c>
       <c r="AC173" s="4" t="n">
-        <v>63.77</v>
+        <v>63.92</v>
       </c>
       <c r="AD173" s="4" t="n">
         <v>0</v>
@@ -22229,7 +22229,7 @@
         </is>
       </c>
       <c r="I210" s="4" t="n">
-        <v>-7.57</v>
+        <v>-7.6</v>
       </c>
       <c r="J210" s="4" t="n">
         <v>10.7</v>
@@ -22286,10 +22286,10 @@
         <v>0</v>
       </c>
       <c r="AB210" s="4" t="n">
-        <v>46.21</v>
+        <v>46.2</v>
       </c>
       <c r="AC210" s="4" t="n">
-        <v>53.79</v>
+        <v>53.8</v>
       </c>
       <c r="AD210" s="4" t="n">
         <v>0</v>
@@ -22945,7 +22945,7 @@
         </is>
       </c>
       <c r="I217" s="4" t="n">
-        <v>24.01</v>
+        <v>24.03</v>
       </c>
       <c r="J217" s="4" t="n">
         <v>99.90000000000001</v>
@@ -22959,13 +22959,13 @@
         </is>
       </c>
       <c r="M217" s="4" t="n">
-        <v>17.34</v>
+        <v>17.35</v>
       </c>
       <c r="N217" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O217" s="4" t="n">
-        <v>24.01</v>
+        <v>24.03</v>
       </c>
       <c r="P217" s="4" t="n">
         <v>0</v>
@@ -23047,7 +23047,7 @@
         </is>
       </c>
       <c r="I218" s="4" t="n">
-        <v>33.63</v>
+        <v>33.64</v>
       </c>
       <c r="J218" s="4" t="n">
         <v>100</v>
@@ -23061,13 +23061,13 @@
         </is>
       </c>
       <c r="M218" s="4" t="n">
-        <v>27.29</v>
+        <v>27.3</v>
       </c>
       <c r="N218" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O218" s="4" t="n">
-        <v>33.63</v>
+        <v>33.64</v>
       </c>
       <c r="P218" s="4" t="n">
         <v>0</v>
@@ -23149,7 +23149,7 @@
         </is>
       </c>
       <c r="I219" s="4" t="n">
-        <v>32.19</v>
+        <v>32.2</v>
       </c>
       <c r="J219" s="4" t="n">
         <v>100</v>
@@ -23163,13 +23163,13 @@
         </is>
       </c>
       <c r="M219" s="4" t="n">
-        <v>22.79</v>
+        <v>22.8</v>
       </c>
       <c r="N219" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O219" s="4" t="n">
-        <v>32.19</v>
+        <v>32.2</v>
       </c>
       <c r="P219" s="4" t="n">
         <v>2.52</v>
@@ -23200,10 +23200,10 @@
         <v>0</v>
       </c>
       <c r="AB219" s="4" t="n">
-        <v>66.09</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AC219" s="4" t="n">
-        <v>33.91</v>
+        <v>33.9</v>
       </c>
       <c r="AD219" s="4" t="n">
         <v>0</v>
@@ -23251,7 +23251,7 @@
         </is>
       </c>
       <c r="I220" s="4" t="n">
-        <v>29.69</v>
+        <v>29.7</v>
       </c>
       <c r="J220" s="4" t="n">
         <v>100</v>
@@ -23265,13 +23265,13 @@
         </is>
       </c>
       <c r="M220" s="4" t="n">
-        <v>23.61</v>
+        <v>23.62</v>
       </c>
       <c r="N220" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O220" s="4" t="n">
-        <v>29.69</v>
+        <v>29.7</v>
       </c>
       <c r="P220" s="4" t="n">
         <v>0</v>
@@ -23302,10 +23302,10 @@
         <v>0</v>
       </c>
       <c r="AB220" s="4" t="n">
-        <v>64.84</v>
+        <v>64.84999999999999</v>
       </c>
       <c r="AC220" s="4" t="n">
-        <v>35.16</v>
+        <v>35.15</v>
       </c>
       <c r="AD220" s="4" t="n">
         <v>0</v>
@@ -23353,7 +23353,7 @@
         </is>
       </c>
       <c r="I221" s="4" t="n">
-        <v>55.31</v>
+        <v>55.32</v>
       </c>
       <c r="J221" s="4" t="n">
         <v>100</v>
@@ -23367,13 +23367,13 @@
         </is>
       </c>
       <c r="M221" s="4" t="n">
-        <v>48.97</v>
+        <v>48.98</v>
       </c>
       <c r="N221" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O221" s="4" t="n">
-        <v>55.31</v>
+        <v>55.32</v>
       </c>
       <c r="P221" s="4" t="n">
         <v>0</v>
@@ -23404,10 +23404,10 @@
         <v>0</v>
       </c>
       <c r="AB221" s="4" t="n">
-        <v>77.65000000000001</v>
+        <v>77.66</v>
       </c>
       <c r="AC221" s="4" t="n">
-        <v>22.35</v>
+        <v>22.34</v>
       </c>
       <c r="AD221" s="4" t="n">
         <v>0</v>
@@ -23451,7 +23451,7 @@
         </is>
       </c>
       <c r="I222" s="4" t="n">
-        <v>28.45</v>
+        <v>28.46</v>
       </c>
       <c r="J222" s="4" t="n">
         <v>100</v>
@@ -23465,13 +23465,13 @@
         </is>
       </c>
       <c r="M222" s="4" t="n">
-        <v>23.82</v>
+        <v>23.83</v>
       </c>
       <c r="N222" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O222" s="4" t="n">
-        <v>28.45</v>
+        <v>28.46</v>
       </c>
       <c r="P222" s="4" t="n">
         <v>0</v>
@@ -23502,10 +23502,10 @@
         <v>0</v>
       </c>
       <c r="AB222" s="4" t="n">
-        <v>64.22</v>
+        <v>64.23</v>
       </c>
       <c r="AC222" s="4" t="n">
-        <v>35.78</v>
+        <v>35.77</v>
       </c>
       <c r="AD222" s="4" t="n">
         <v>0</v>
@@ -23553,7 +23553,7 @@
         </is>
       </c>
       <c r="I223" s="4" t="n">
-        <v>76.09999999999999</v>
+        <v>76.11</v>
       </c>
       <c r="J223" s="4" t="n">
         <v>100</v>
@@ -23567,13 +23567,13 @@
         </is>
       </c>
       <c r="M223" s="4" t="n">
-        <v>68.98</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="N223" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O223" s="4" t="n">
-        <v>76.09999999999999</v>
+        <v>76.11</v>
       </c>
       <c r="P223" s="4" t="n">
         <v>0</v>
@@ -23604,10 +23604,10 @@
         <v>0</v>
       </c>
       <c r="AB223" s="4" t="n">
-        <v>88.05</v>
+        <v>88.06</v>
       </c>
       <c r="AC223" s="4" t="n">
-        <v>11.95</v>
+        <v>11.94</v>
       </c>
       <c r="AD223" s="4" t="n">
         <v>0</v>
@@ -23655,7 +23655,7 @@
         </is>
       </c>
       <c r="I224" s="4" t="n">
-        <v>45.42</v>
+        <v>45.43</v>
       </c>
       <c r="J224" s="4" t="n">
         <v>100</v>
@@ -23669,13 +23669,13 @@
         </is>
       </c>
       <c r="M224" s="4" t="n">
-        <v>30.38</v>
+        <v>30.4</v>
       </c>
       <c r="N224" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O224" s="4" t="n">
-        <v>45.42</v>
+        <v>45.43</v>
       </c>
       <c r="P224" s="4" t="n">
         <v>0</v>
@@ -23757,7 +23757,7 @@
         </is>
       </c>
       <c r="I225" s="4" t="n">
-        <v>22.43</v>
+        <v>22.45</v>
       </c>
       <c r="J225" s="4" t="n">
         <v>99.90000000000001</v>
@@ -23771,13 +23771,13 @@
         </is>
       </c>
       <c r="M225" s="4" t="n">
-        <v>13.86</v>
+        <v>13.87</v>
       </c>
       <c r="N225" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O225" s="4" t="n">
-        <v>22.43</v>
+        <v>22.45</v>
       </c>
       <c r="P225" s="4" t="n">
         <v>0.51</v>
@@ -24667,7 +24667,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.96</v>
+        <v>30.9</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24681,13 +24681,13 @@
         </is>
       </c>
       <c r="M234" s="4" t="n">
-        <v>22.29</v>
+        <v>22.28</v>
       </c>
       <c r="N234" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O234" s="4" t="n">
-        <v>31.25</v>
+        <v>31.24</v>
       </c>
       <c r="P234" s="4" t="n">
         <v>1</v>
@@ -24765,13 +24765,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-3.44</v>
+        <v>-3.84</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>39.6</v>
+        <v>39.7</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>60.4</v>
+        <v>60.3</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -24779,13 +24779,13 @@
         </is>
       </c>
       <c r="M235" s="4" t="n">
-        <v>-8.85</v>
+        <v>-8.859999999999999</v>
       </c>
       <c r="N235" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O235" s="4" t="n">
-        <v>-5.2</v>
+        <v>-5.21</v>
       </c>
       <c r="P235" s="4" t="n">
         <v>-0.48</v>
@@ -24822,10 +24822,10 @@
         <v>0</v>
       </c>
       <c r="AB235" s="4" t="n">
-        <v>45.47</v>
+        <v>45.46</v>
       </c>
       <c r="AC235" s="4" t="n">
-        <v>49.53</v>
+        <v>49.54</v>
       </c>
       <c r="AD235" s="4" t="n">
         <v>5</v>
@@ -24873,7 +24873,7 @@
         </is>
       </c>
       <c r="I236" s="4" t="n">
-        <v>-12.78</v>
+        <v>-12.77</v>
       </c>
       <c r="J236" s="4" t="n">
         <v>1</v>
@@ -24887,13 +24887,13 @@
         </is>
       </c>
       <c r="M236" s="4" t="n">
-        <v>-17.27</v>
+        <v>-17.26</v>
       </c>
       <c r="N236" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O236" s="4" t="n">
-        <v>-12.78</v>
+        <v>-12.77</v>
       </c>
       <c r="P236" s="4" t="n">
         <v>-0.61</v>
@@ -25199,7 +25199,7 @@
         <v>5.13</v>
       </c>
       <c r="O239" s="4" t="n">
-        <v>-2.07</v>
+        <v>-2.06</v>
       </c>
       <c r="P239" s="4" t="n">
         <v>-0.31</v>
@@ -25301,7 +25301,7 @@
         </is>
       </c>
       <c r="M240" s="4" t="n">
-        <v>-22.64</v>
+        <v>-22.63</v>
       </c>
       <c r="N240" s="4" t="n">
         <v>5.13</v>
@@ -25491,13 +25491,13 @@
         </is>
       </c>
       <c r="I242" s="4" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="J242" s="4" t="n">
-        <v>65.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="K242" s="4" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="L242" t="inlineStr">
         <is>
@@ -25511,7 +25511,7 @@
         <v>5.13</v>
       </c>
       <c r="O242" s="4" t="n">
-        <v>3.09</v>
+        <v>3.1</v>
       </c>
       <c r="P242" s="4" t="n">
         <v>-0.62</v>
@@ -25548,10 +25548,10 @@
         <v>0</v>
       </c>
       <c r="AB242" s="4" t="n">
-        <v>50.43</v>
+        <v>50.44</v>
       </c>
       <c r="AC242" s="4" t="n">
-        <v>49.57</v>
+        <v>49.56</v>
       </c>
       <c r="AD242" s="4" t="n">
         <v>0</v>
@@ -25715,7 +25715,7 @@
         </is>
       </c>
       <c r="M244" s="4" t="n">
-        <v>-28.17</v>
+        <v>-28.16</v>
       </c>
       <c r="N244" s="4" t="n">
         <v>5.13</v>
@@ -25799,7 +25799,7 @@
         </is>
       </c>
       <c r="I245" s="4" t="n">
-        <v>2.31</v>
+        <v>2.32</v>
       </c>
       <c r="J245" s="4" t="n">
         <v>70.90000000000001</v>
@@ -25903,7 +25903,7 @@
         </is>
       </c>
       <c r="I246" s="4" t="n">
-        <v>27.77</v>
+        <v>27.78</v>
       </c>
       <c r="J246" s="4" t="n">
         <v>100</v>
@@ -25923,7 +25923,7 @@
         <v>5.13</v>
       </c>
       <c r="O246" s="4" t="n">
-        <v>27.77</v>
+        <v>27.78</v>
       </c>
       <c r="P246" s="4" t="n">
         <v>2.12</v>
@@ -26005,7 +26005,7 @@
         </is>
       </c>
       <c r="I247" s="4" t="n">
-        <v>56.32</v>
+        <v>56.33</v>
       </c>
       <c r="J247" s="4" t="n">
         <v>100</v>
@@ -26019,13 +26019,13 @@
         </is>
       </c>
       <c r="M247" s="4" t="n">
-        <v>46.21</v>
+        <v>46.22</v>
       </c>
       <c r="N247" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O247" s="4" t="n">
-        <v>56.32</v>
+        <v>56.33</v>
       </c>
       <c r="P247" s="4" t="n">
         <v>0</v>
@@ -26209,7 +26209,7 @@
         </is>
       </c>
       <c r="I249" s="4" t="n">
-        <v>-6.12</v>
+        <v>-6.13</v>
       </c>
       <c r="J249" s="4" t="n">
         <v>15.3</v>
@@ -26229,7 +26229,7 @@
         <v>5.13</v>
       </c>
       <c r="O249" s="4" t="n">
-        <v>-6.37</v>
+        <v>-6.38</v>
       </c>
       <c r="P249" s="4" t="n">
         <v>-0.02</v>
@@ -26313,7 +26313,7 @@
         </is>
       </c>
       <c r="I250" s="4" t="n">
-        <v>11.68</v>
+        <v>11.7</v>
       </c>
       <c r="J250" s="4" t="n">
         <v>98.8</v>
@@ -26333,7 +26333,7 @@
         <v>5.13</v>
       </c>
       <c r="O250" s="4" t="n">
-        <v>13.47</v>
+        <v>13.46</v>
       </c>
       <c r="P250" s="4" t="n">
         <v>0.47</v>
@@ -26370,10 +26370,10 @@
         <v>0</v>
       </c>
       <c r="AB250" s="4" t="n">
-        <v>55.84</v>
+        <v>55.85</v>
       </c>
       <c r="AC250" s="4" t="n">
-        <v>44.16</v>
+        <v>44.15</v>
       </c>
       <c r="AD250" s="4" t="n">
         <v>0</v>
@@ -26676,10 +26676,10 @@
         <v>0</v>
       </c>
       <c r="AB253" s="4" t="n">
-        <v>82.90000000000001</v>
+        <v>82.89</v>
       </c>
       <c r="AC253" s="4" t="n">
-        <v>17.1</v>
+        <v>17.11</v>
       </c>
       <c r="AD253" s="4" t="n">
         <v>0</v>
@@ -26727,7 +26727,7 @@
         </is>
       </c>
       <c r="I254" s="4" t="n">
-        <v>-14.68</v>
+        <v>-14.69</v>
       </c>
       <c r="J254" s="4" t="n">
         <v>0.7</v>
@@ -26747,7 +26747,7 @@
         <v>5.13</v>
       </c>
       <c r="O254" s="4" t="n">
-        <v>-14.68</v>
+        <v>-14.69</v>
       </c>
       <c r="P254" s="4" t="n">
         <v>0</v>
@@ -26829,7 +26829,7 @@
         </is>
       </c>
       <c r="I255" s="4" t="n">
-        <v>-31.02</v>
+        <v>-31.03</v>
       </c>
       <c r="J255" s="4" t="n">
         <v>0</v>
@@ -26843,13 +26843,13 @@
         </is>
       </c>
       <c r="M255" s="4" t="n">
-        <v>-33.64</v>
+        <v>-33.65</v>
       </c>
       <c r="N255" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O255" s="4" t="n">
-        <v>-31.02</v>
+        <v>-31.03</v>
       </c>
       <c r="P255" s="4" t="n">
         <v>0</v>
@@ -26931,7 +26931,7 @@
         </is>
       </c>
       <c r="I256" s="4" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="J256" s="4" t="n">
         <v>7.5</v>
@@ -26951,7 +26951,7 @@
         <v>5.13</v>
       </c>
       <c r="O256" s="4" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.710000000000001</v>
       </c>
       <c r="P256" s="4" t="n">
         <v>0</v>
@@ -27135,7 +27135,7 @@
         </is>
       </c>
       <c r="I258" s="4" t="n">
-        <v>-10.61</v>
+        <v>-10.63</v>
       </c>
       <c r="J258" s="4" t="n">
         <v>2.7</v>
@@ -27192,10 +27192,10 @@
         <v>0</v>
       </c>
       <c r="AB258" s="4" t="n">
-        <v>44.69</v>
+        <v>44.68</v>
       </c>
       <c r="AC258" s="4" t="n">
-        <v>55.31</v>
+        <v>55.32</v>
       </c>
       <c r="AD258" s="4" t="n">
         <v>0</v>
@@ -28255,13 +28255,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-5.9</v>
+        <v>-5.94</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>16.1</v>
+        <v>15.9</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>83.90000000000001</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28269,13 +28269,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-11.02</v>
+        <v>-11.07</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-7.02</v>
+        <v>-7.06</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28312,10 +28312,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>47.05</v>
+        <v>47.03</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>52.95</v>
+        <v>52.97</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28363,7 +28363,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-32.75</v>
+        <v>-32.8</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28377,13 +28377,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-29.98</v>
+        <v>-30.03</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-32.75</v>
+        <v>-32.8</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28414,10 +28414,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.62</v>
+        <v>33.6</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.38</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -28675,7 +28675,7 @@
         </is>
       </c>
       <c r="I273" s="4" t="n">
-        <v>-8.1</v>
+        <v>-8.109999999999999</v>
       </c>
       <c r="J273" s="4" t="n">
         <v>9.199999999999999</v>
@@ -28689,13 +28689,13 @@
         </is>
       </c>
       <c r="M273" s="4" t="n">
-        <v>-9.91</v>
+        <v>-9.92</v>
       </c>
       <c r="N273" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O273" s="4" t="n">
-        <v>-8.1</v>
+        <v>-8.109999999999999</v>
       </c>
       <c r="P273" s="4" t="n">
         <v>-1.57</v>
@@ -28791,7 +28791,7 @@
         </is>
       </c>
       <c r="M274" s="4" t="n">
-        <v>48.6</v>
+        <v>48.59</v>
       </c>
       <c r="N274" s="4" t="n">
         <v>5.13</v>
@@ -29199,7 +29199,7 @@
         </is>
       </c>
       <c r="M278" s="4" t="n">
-        <v>-16.99</v>
+        <v>-17</v>
       </c>
       <c r="N278" s="4" t="n">
         <v>5.13</v>
@@ -29338,10 +29338,10 @@
         <v>0</v>
       </c>
       <c r="AB279" s="4" t="n">
-        <v>44.18</v>
+        <v>44.17</v>
       </c>
       <c r="AC279" s="4" t="n">
-        <v>55.82</v>
+        <v>55.83</v>
       </c>
       <c r="AD279" s="4" t="n">
         <v>0</v>
@@ -29511,7 +29511,7 @@
         </is>
       </c>
       <c r="M281" s="4" t="n">
-        <v>-7.93</v>
+        <v>-7.94</v>
       </c>
       <c r="N281" s="4" t="n">
         <v>5.13</v>
@@ -29727,7 +29727,7 @@
         <v>5.13</v>
       </c>
       <c r="O283" s="4" t="n">
-        <v>-13.17</v>
+        <v>-13.18</v>
       </c>
       <c r="P283" s="4" t="n">
         <v>-0.19</v>
@@ -29809,7 +29809,7 @@
         </is>
       </c>
       <c r="I284" s="4" t="n">
-        <v>-13.12</v>
+        <v>-13.13</v>
       </c>
       <c r="J284" s="4" t="n">
         <v>0.9</v>
@@ -30019,13 +30019,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.68</v>
+        <v>-9.76</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>95.09999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -30033,13 +30033,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.94</v>
+        <v>-9.029999999999999</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-10.3</v>
+        <v>-10.39</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30076,10 +30076,10 @@
         <v>0</v>
       </c>
       <c r="AB286" s="4" t="n">
-        <v>45.16</v>
+        <v>45.12</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>54.84</v>
+        <v>54.88</v>
       </c>
       <c r="AD286" s="4" t="n">
         <v>0</v>
@@ -30123,7 +30123,7 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>12.45</v>
+        <v>12.38</v>
       </c>
       <c r="J287" s="4" t="n">
         <v>98.90000000000001</v>
@@ -30137,13 +30137,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>8.92</v>
+        <v>8.83</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.12</v>
+        <v>14.03</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30180,10 +30180,10 @@
         <v>0</v>
       </c>
       <c r="AB287" s="4" t="n">
-        <v>56.22</v>
+        <v>56.19</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>43.78</v>
+        <v>43.81</v>
       </c>
       <c r="AD287" s="4" t="n">
         <v>0</v>
@@ -30231,7 +30231,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.85</v>
+        <v>-52.94</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30245,13 +30245,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.89</v>
+        <v>-49.98</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.85</v>
+        <v>-52.94</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30282,10 +30282,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.57</v>
+        <v>23.53</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.43000000000001</v>
+        <v>76.47</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -31157,7 +31157,7 @@
         </is>
       </c>
       <c r="I297" s="4" t="n">
-        <v>4.48</v>
+        <v>4.49</v>
       </c>
       <c r="J297" s="4" t="n">
         <v>79</v>
@@ -31771,7 +31771,7 @@
         </is>
       </c>
       <c r="I303" s="4" t="n">
-        <v>25.8</v>
+        <v>25.81</v>
       </c>
       <c r="J303" s="4" t="n">
         <v>100</v>
@@ -31785,13 +31785,13 @@
         </is>
       </c>
       <c r="M303" s="4" t="n">
-        <v>15.79</v>
+        <v>15.8</v>
       </c>
       <c r="N303" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O303" s="4" t="n">
-        <v>25.8</v>
+        <v>25.81</v>
       </c>
       <c r="P303" s="4" t="n">
         <v>1.68</v>
@@ -31822,10 +31822,10 @@
         <v>0</v>
       </c>
       <c r="AB303" s="4" t="n">
-        <v>62.9</v>
+        <v>62.91</v>
       </c>
       <c r="AC303" s="4" t="n">
-        <v>37.1</v>
+        <v>37.09</v>
       </c>
       <c r="AD303" s="4" t="n">
         <v>0</v>
@@ -31873,7 +31873,7 @@
         </is>
       </c>
       <c r="I304" s="4" t="n">
-        <v>14.2</v>
+        <v>14.22</v>
       </c>
       <c r="J304" s="4" t="n">
         <v>99.2</v>
@@ -31887,13 +31887,13 @@
         </is>
       </c>
       <c r="M304" s="4" t="n">
-        <v>2.94</v>
+        <v>2.95</v>
       </c>
       <c r="N304" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O304" s="4" t="n">
-        <v>16.22</v>
+        <v>16.23</v>
       </c>
       <c r="P304" s="4" t="n">
         <v>0.67</v>
@@ -31930,10 +31930,10 @@
         <v>0</v>
       </c>
       <c r="AB304" s="4" t="n">
-        <v>57.1</v>
+        <v>57.11</v>
       </c>
       <c r="AC304" s="4" t="n">
-        <v>42.9</v>
+        <v>42.89</v>
       </c>
       <c r="AD304" s="4" t="n">
         <v>0</v>
@@ -31981,7 +31981,7 @@
         </is>
       </c>
       <c r="I305" s="4" t="n">
-        <v>22.82</v>
+        <v>22.83</v>
       </c>
       <c r="J305" s="4" t="n">
         <v>99.90000000000001</v>
@@ -31995,13 +31995,13 @@
         </is>
       </c>
       <c r="M305" s="4" t="n">
-        <v>9.550000000000001</v>
+        <v>9.56</v>
       </c>
       <c r="N305" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O305" s="4" t="n">
-        <v>22.82</v>
+        <v>22.83</v>
       </c>
       <c r="P305" s="4" t="n">
         <v>0.73</v>
@@ -32083,7 +32083,7 @@
         </is>
       </c>
       <c r="I306" s="4" t="n">
-        <v>16.18</v>
+        <v>16.19</v>
       </c>
       <c r="J306" s="4" t="n">
         <v>99.5</v>
@@ -32103,7 +32103,7 @@
         <v>5.13</v>
       </c>
       <c r="O306" s="4" t="n">
-        <v>16.18</v>
+        <v>16.19</v>
       </c>
       <c r="P306" s="4" t="n">
         <v>-0.16</v>
@@ -32181,13 +32181,13 @@
         </is>
       </c>
       <c r="I307" s="4" t="n">
-        <v>-3.63</v>
+        <v>-3.72</v>
       </c>
       <c r="J307" s="4" t="n">
-        <v>24.1</v>
+        <v>23.8</v>
       </c>
       <c r="K307" s="4" t="n">
-        <v>75.90000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -32195,13 +32195,13 @@
         </is>
       </c>
       <c r="M307" s="4" t="n">
-        <v>-12.43</v>
+        <v>-12.42</v>
       </c>
       <c r="N307" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O307" s="4" t="n">
-        <v>-8.630000000000001</v>
+        <v>-8.619999999999999</v>
       </c>
       <c r="P307" s="4" t="n">
         <v>-1.32</v>
@@ -32238,10 +32238,10 @@
         <v>0</v>
       </c>
       <c r="AB307" s="4" t="n">
-        <v>48.18</v>
+        <v>48.14</v>
       </c>
       <c r="AC307" s="4" t="n">
-        <v>51.82</v>
+        <v>51.86</v>
       </c>
       <c r="AD307" s="4" t="n">
         <v>0</v>
@@ -32289,7 +32289,7 @@
         </is>
       </c>
       <c r="I308" s="4" t="n">
-        <v>11.65</v>
+        <v>11.66</v>
       </c>
       <c r="J308" s="4" t="n">
         <v>98.8</v>
@@ -32303,13 +32303,13 @@
         </is>
       </c>
       <c r="M308" s="4" t="n">
-        <v>2.5</v>
+        <v>2.51</v>
       </c>
       <c r="N308" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O308" s="4" t="n">
-        <v>11.65</v>
+        <v>11.66</v>
       </c>
       <c r="P308" s="4" t="n">
         <v>0.06</v>
@@ -32391,7 +32391,7 @@
         </is>
       </c>
       <c r="I309" s="4" t="n">
-        <v>17.44</v>
+        <v>17.45</v>
       </c>
       <c r="J309" s="4" t="n">
         <v>99.59999999999999</v>
@@ -32405,13 +32405,13 @@
         </is>
       </c>
       <c r="M309" s="4" t="n">
-        <v>5.43</v>
+        <v>5.44</v>
       </c>
       <c r="N309" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O309" s="4" t="n">
-        <v>17.44</v>
+        <v>17.45</v>
       </c>
       <c r="P309" s="4" t="n">
         <v>0.97</v>
@@ -34121,13 +34121,13 @@
         </is>
       </c>
       <c r="I326" s="4" t="n">
-        <v>2.3</v>
+        <v>2.32</v>
       </c>
       <c r="J326" s="4" t="n">
-        <v>70.8</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K326" s="4" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -34178,10 +34178,10 @@
         <v>0</v>
       </c>
       <c r="AB326" s="4" t="n">
-        <v>51.15</v>
+        <v>51.16</v>
       </c>
       <c r="AC326" s="4" t="n">
-        <v>48.85</v>
+        <v>48.84</v>
       </c>
       <c r="AD326" s="4" t="n">
         <v>0</v>
@@ -34537,7 +34537,7 @@
         </is>
       </c>
       <c r="I330" s="4" t="n">
-        <v>-12.53</v>
+        <v>-12.57</v>
       </c>
       <c r="J330" s="4" t="n">
         <v>1</v>
@@ -34594,10 +34594,10 @@
         <v>0</v>
       </c>
       <c r="AB330" s="4" t="n">
-        <v>43.73</v>
+        <v>43.72</v>
       </c>
       <c r="AC330" s="4" t="n">
-        <v>56.27</v>
+        <v>56.28</v>
       </c>
       <c r="AD330" s="4" t="n">
         <v>0</v>
@@ -35155,7 +35155,7 @@
         </is>
       </c>
       <c r="I336" s="4" t="n">
-        <v>11.64</v>
+        <v>11.63</v>
       </c>
       <c r="J336" s="4" t="n">
         <v>98.8</v>
@@ -35169,13 +35169,13 @@
         </is>
       </c>
       <c r="M336" s="4" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
       <c r="N336" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O336" s="4" t="n">
-        <v>11.64</v>
+        <v>11.63</v>
       </c>
       <c r="P336" s="4" t="n">
         <v>0.77</v>
@@ -35308,10 +35308,10 @@
         <v>0</v>
       </c>
       <c r="AB337" s="4" t="n">
-        <v>31.85</v>
+        <v>31.84</v>
       </c>
       <c r="AC337" s="4" t="n">
-        <v>68.15000000000001</v>
+        <v>68.16</v>
       </c>
       <c r="AD337" s="4" t="n">
         <v>0</v>
@@ -35359,7 +35359,7 @@
         </is>
       </c>
       <c r="I338" s="4" t="n">
-        <v>52.59</v>
+        <v>52.58</v>
       </c>
       <c r="J338" s="4" t="n">
         <v>100</v>
@@ -35379,7 +35379,7 @@
         <v>5.13</v>
       </c>
       <c r="O338" s="4" t="n">
-        <v>52.59</v>
+        <v>52.58</v>
       </c>
       <c r="P338" s="4" t="n">
         <v>0</v>
@@ -35461,7 +35461,7 @@
         </is>
       </c>
       <c r="I339" s="4" t="n">
-        <v>-38.7</v>
+        <v>-38.71</v>
       </c>
       <c r="J339" s="4" t="n">
         <v>0</v>
@@ -35481,7 +35481,7 @@
         <v>5.13</v>
       </c>
       <c r="O339" s="4" t="n">
-        <v>-38.7</v>
+        <v>-38.71</v>
       </c>
       <c r="P339" s="4" t="n">
         <v>-3.15</v>
@@ -35577,7 +35577,7 @@
         </is>
       </c>
       <c r="M340" s="4" t="n">
-        <v>-19.28</v>
+        <v>-19.29</v>
       </c>
       <c r="N340" s="4" t="n">
         <v>5.13</v>
@@ -35767,13 +35767,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>-6.61</v>
+        <v>-6.63</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>13.7</v>
+        <v>13.6</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>86.3</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35824,10 +35824,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>46.69</v>
+        <v>46.68</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>53.31</v>
+        <v>53.32</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -35926,10 +35926,10 @@
         <v>0</v>
       </c>
       <c r="AB343" s="4" t="n">
-        <v>45.6</v>
+        <v>45.59</v>
       </c>
       <c r="AC343" s="4" t="n">
-        <v>54.4</v>
+        <v>54.41</v>
       </c>
       <c r="AD343" s="4" t="n">
         <v>0</v>
@@ -35977,7 +35977,7 @@
         </is>
       </c>
       <c r="I344" s="4" t="n">
-        <v>9.18</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J344" s="4" t="n">
         <v>93.8</v>
@@ -35991,7 +35991,7 @@
         </is>
       </c>
       <c r="M344" s="4" t="n">
-        <v>-5.63</v>
+        <v>-5.64</v>
       </c>
       <c r="N344" s="4" t="n">
         <v>5.13</v>
@@ -36034,10 +36034,10 @@
         <v>0</v>
       </c>
       <c r="AB344" s="4" t="n">
-        <v>54.59</v>
+        <v>54.6</v>
       </c>
       <c r="AC344" s="4" t="n">
-        <v>45.41</v>
+        <v>45.4</v>
       </c>
       <c r="AD344" s="4" t="n">
         <v>0</v>
@@ -36085,13 +36085,13 @@
         </is>
       </c>
       <c r="I345" s="4" t="n">
-        <v>-8</v>
+        <v>-8.029999999999999</v>
       </c>
       <c r="J345" s="4" t="n">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="K345" s="4" t="n">
-        <v>90.5</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="L345" t="inlineStr">
         <is>
@@ -36142,10 +36142,10 @@
         <v>0</v>
       </c>
       <c r="AB345" s="4" t="n">
-        <v>46</v>
+        <v>45.98</v>
       </c>
       <c r="AC345" s="4" t="n">
-        <v>54</v>
+        <v>54.02</v>
       </c>
       <c r="AD345" s="4" t="n">
         <v>0</v>
@@ -36193,7 +36193,7 @@
         </is>
       </c>
       <c r="I346" s="4" t="n">
-        <v>70.48999999999999</v>
+        <v>70.48</v>
       </c>
       <c r="J346" s="4" t="n">
         <v>100</v>
@@ -36207,13 +36207,13 @@
         </is>
       </c>
       <c r="M346" s="4" t="n">
-        <v>60.42</v>
+        <v>60.41</v>
       </c>
       <c r="N346" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O346" s="4" t="n">
-        <v>70.48999999999999</v>
+        <v>70.48</v>
       </c>
       <c r="P346" s="4" t="n">
         <v>0</v>
@@ -36295,7 +36295,7 @@
         </is>
       </c>
       <c r="I347" s="4" t="n">
-        <v>-25.88</v>
+        <v>-25.89</v>
       </c>
       <c r="J347" s="4" t="n">
         <v>0</v>
@@ -36309,13 +36309,13 @@
         </is>
       </c>
       <c r="M347" s="4" t="n">
-        <v>-26.34</v>
+        <v>-26.35</v>
       </c>
       <c r="N347" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O347" s="4" t="n">
-        <v>-25.88</v>
+        <v>-25.89</v>
       </c>
       <c r="P347" s="4" t="n">
         <v>-1.94</v>
@@ -36411,7 +36411,7 @@
         </is>
       </c>
       <c r="M348" s="4" t="n">
-        <v>7.92</v>
+        <v>7.91</v>
       </c>
       <c r="N348" s="4" t="n">
         <v>5.13</v>
@@ -36513,7 +36513,7 @@
         </is>
       </c>
       <c r="M349" s="4" t="n">
-        <v>-15.7</v>
+        <v>-15.71</v>
       </c>
       <c r="N349" s="4" t="n">
         <v>5.13</v>
@@ -36652,10 +36652,10 @@
         <v>0</v>
       </c>
       <c r="AB350" s="4" t="n">
-        <v>47.08</v>
+        <v>47.07</v>
       </c>
       <c r="AC350" s="4" t="n">
-        <v>52.92</v>
+        <v>52.93</v>
       </c>
       <c r="AD350" s="4" t="n">
         <v>0</v>
@@ -37209,7 +37209,7 @@
         </is>
       </c>
       <c r="I356" s="4" t="n">
-        <v>49.25</v>
+        <v>49.26</v>
       </c>
       <c r="J356" s="4" t="n">
         <v>100</v>
@@ -37223,13 +37223,13 @@
         </is>
       </c>
       <c r="M356" s="4" t="n">
-        <v>38.57</v>
+        <v>38.58</v>
       </c>
       <c r="N356" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O356" s="4" t="n">
-        <v>49.25</v>
+        <v>49.26</v>
       </c>
       <c r="P356" s="4" t="n">
         <v>2.08</v>
@@ -37325,7 +37325,7 @@
         </is>
       </c>
       <c r="M357" s="4" t="n">
-        <v>-28.25</v>
+        <v>-28.24</v>
       </c>
       <c r="N357" s="4" t="n">
         <v>5.13</v>
@@ -37413,7 +37413,7 @@
         </is>
       </c>
       <c r="I358" s="4" t="n">
-        <v>54.96</v>
+        <v>54.97</v>
       </c>
       <c r="J358" s="4" t="n">
         <v>100</v>
@@ -37433,7 +37433,7 @@
         <v>5.13</v>
       </c>
       <c r="O358" s="4" t="n">
-        <v>54.96</v>
+        <v>54.97</v>
       </c>
       <c r="P358" s="4" t="n">
         <v>0</v>
@@ -37515,7 +37515,7 @@
         </is>
       </c>
       <c r="I359" s="4" t="n">
-        <v>16.8</v>
+        <v>16.81</v>
       </c>
       <c r="J359" s="4" t="n">
         <v>99.5</v>
@@ -37529,13 +37529,13 @@
         </is>
       </c>
       <c r="M359" s="4" t="n">
-        <v>11.65</v>
+        <v>11.66</v>
       </c>
       <c r="N359" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O359" s="4" t="n">
-        <v>16.8</v>
+        <v>16.81</v>
       </c>
       <c r="P359" s="4" t="n">
         <v>0.47</v>
@@ -37733,7 +37733,7 @@
         </is>
       </c>
       <c r="M361" s="4" t="n">
-        <v>11.1</v>
+        <v>11.11</v>
       </c>
       <c r="N361" s="4" t="n">
         <v>5.13</v>
@@ -37770,10 +37770,10 @@
         <v>0</v>
       </c>
       <c r="AB361" s="4" t="n">
-        <v>58.89</v>
+        <v>58.9</v>
       </c>
       <c r="AC361" s="4" t="n">
-        <v>41.11</v>
+        <v>41.1</v>
       </c>
       <c r="AD361" s="4" t="n">
         <v>0</v>
@@ -37821,7 +37821,7 @@
         </is>
       </c>
       <c r="I362" s="4" t="n">
-        <v>-2.16</v>
+        <v>-2.15</v>
       </c>
       <c r="J362" s="4" t="n">
         <v>29.8</v>
@@ -38435,7 +38435,7 @@
         </is>
       </c>
       <c r="I368" s="4" t="n">
-        <v>2.26</v>
+        <v>2.28</v>
       </c>
       <c r="J368" s="4" t="n">
         <v>70.7</v>
@@ -38492,10 +38492,10 @@
         <v>0</v>
       </c>
       <c r="AB368" s="4" t="n">
-        <v>51.13</v>
+        <v>51.14</v>
       </c>
       <c r="AC368" s="4" t="n">
-        <v>48.87</v>
+        <v>48.86</v>
       </c>
       <c r="AD368" s="4" t="n">
         <v>0</v>
@@ -38747,7 +38747,7 @@
         </is>
       </c>
       <c r="I371" s="4" t="n">
-        <v>8.67</v>
+        <v>8.68</v>
       </c>
       <c r="J371" s="4" t="n">
         <v>92.40000000000001</v>
@@ -39569,7 +39569,7 @@
         </is>
       </c>
       <c r="I379" s="4" t="n">
-        <v>40.38</v>
+        <v>40.39</v>
       </c>
       <c r="J379" s="4" t="n">
         <v>100</v>
@@ -39583,13 +39583,13 @@
         </is>
       </c>
       <c r="M379" s="4" t="n">
-        <v>27.1</v>
+        <v>27.11</v>
       </c>
       <c r="N379" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O379" s="4" t="n">
-        <v>40.38</v>
+        <v>40.39</v>
       </c>
       <c r="P379" s="4" t="n">
         <v>0</v>
@@ -39620,10 +39620,10 @@
         <v>0</v>
       </c>
       <c r="AB379" s="4" t="n">
-        <v>70.19</v>
+        <v>70.2</v>
       </c>
       <c r="AC379" s="4" t="n">
-        <v>29.81</v>
+        <v>29.8</v>
       </c>
       <c r="AD379" s="4" t="n">
         <v>0</v>
@@ -39671,7 +39671,7 @@
         </is>
       </c>
       <c r="I380" s="4" t="n">
-        <v>17.09</v>
+        <v>17.1</v>
       </c>
       <c r="J380" s="4" t="n">
         <v>99.59999999999999</v>
@@ -39685,13 +39685,13 @@
         </is>
       </c>
       <c r="M380" s="4" t="n">
-        <v>11.24</v>
+        <v>11.25</v>
       </c>
       <c r="N380" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O380" s="4" t="n">
-        <v>17.09</v>
+        <v>17.1</v>
       </c>
       <c r="P380" s="4" t="n">
         <v>-0.61</v>
@@ -40985,7 +40985,7 @@
         </is>
       </c>
       <c r="I393" s="4" t="n">
-        <v>-13.73</v>
+        <v>-13.74</v>
       </c>
       <c r="J393" s="4" t="n">
         <v>0.8</v>
@@ -41507,7 +41507,7 @@
         </is>
       </c>
       <c r="M398" s="4" t="n">
-        <v>-44.68</v>
+        <v>-44.69</v>
       </c>
       <c r="N398" s="4" t="n">
         <v>5.13</v>
@@ -41693,7 +41693,7 @@
         </is>
       </c>
       <c r="I400" s="4" t="n">
-        <v>-16.08</v>
+        <v>-16.09</v>
       </c>
       <c r="J400" s="4" t="n">
         <v>0.5</v>
@@ -41707,13 +41707,13 @@
         </is>
       </c>
       <c r="M400" s="4" t="n">
-        <v>-19.28</v>
+        <v>-19.29</v>
       </c>
       <c r="N400" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O400" s="4" t="n">
-        <v>-16.08</v>
+        <v>-16.09</v>
       </c>
       <c r="P400" s="4" t="n">
         <v>-0.25</v>
@@ -41897,7 +41897,7 @@
         </is>
       </c>
       <c r="I402" s="4" t="n">
-        <v>-14.04</v>
+        <v>-14.05</v>
       </c>
       <c r="J402" s="4" t="n">
         <v>0.8</v>
@@ -41917,7 +41917,7 @@
         <v>5.13</v>
       </c>
       <c r="O402" s="4" t="n">
-        <v>-14.04</v>
+        <v>-14.05</v>
       </c>
       <c r="P402" s="4" t="n">
         <v>-2.23</v>
@@ -41999,7 +41999,7 @@
         </is>
       </c>
       <c r="I403" s="4" t="n">
-        <v>-19.42</v>
+        <v>-19.43</v>
       </c>
       <c r="J403" s="4" t="n">
         <v>0.3</v>
@@ -42019,7 +42019,7 @@
         <v>5.13</v>
       </c>
       <c r="O403" s="4" t="n">
-        <v>-19.42</v>
+        <v>-19.43</v>
       </c>
       <c r="P403" s="4" t="n">
         <v>-2.94</v>
@@ -42101,7 +42101,7 @@
         </is>
       </c>
       <c r="I404" s="4" t="n">
-        <v>40.34</v>
+        <v>40.33</v>
       </c>
       <c r="J404" s="4" t="n">
         <v>100</v>
@@ -42121,7 +42121,7 @@
         <v>5.13</v>
       </c>
       <c r="O404" s="4" t="n">
-        <v>40.34</v>
+        <v>40.33</v>
       </c>
       <c r="P404" s="4" t="n">
         <v>1.84</v>
@@ -42297,7 +42297,7 @@
         </is>
       </c>
       <c r="I406" s="4" t="n">
-        <v>-7.34</v>
+        <v>-7.35</v>
       </c>
       <c r="J406" s="4" t="n">
         <v>11.4</v>
@@ -42317,7 +42317,7 @@
         <v>5.13</v>
       </c>
       <c r="O406" s="4" t="n">
-        <v>-7.34</v>
+        <v>-7.35</v>
       </c>
       <c r="P406" s="4" t="n">
         <v>-1.92</v>
@@ -42395,7 +42395,7 @@
         </is>
       </c>
       <c r="I407" s="4" t="n">
-        <v>-13.73</v>
+        <v>-13.74</v>
       </c>
       <c r="J407" s="4" t="n">
         <v>0.8</v>
@@ -42409,13 +42409,13 @@
         </is>
       </c>
       <c r="M407" s="4" t="n">
-        <v>-17.41</v>
+        <v>-17.42</v>
       </c>
       <c r="N407" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O407" s="4" t="n">
-        <v>-13.73</v>
+        <v>-13.74</v>
       </c>
       <c r="P407" s="4" t="n">
         <v>-1.52</v>
@@ -42497,7 +42497,7 @@
         </is>
       </c>
       <c r="I408" s="4" t="n">
-        <v>-28.09</v>
+        <v>-28.1</v>
       </c>
       <c r="J408" s="4" t="n">
         <v>0</v>
@@ -42511,13 +42511,13 @@
         </is>
       </c>
       <c r="M408" s="4" t="n">
-        <v>-30.1</v>
+        <v>-30.11</v>
       </c>
       <c r="N408" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O408" s="4" t="n">
-        <v>-28.09</v>
+        <v>-28.1</v>
       </c>
       <c r="P408" s="4" t="n">
         <v>-2.36</v>
@@ -42613,7 +42613,7 @@
         </is>
       </c>
       <c r="M409" s="4" t="n">
-        <v>-19.05</v>
+        <v>-19.06</v>
       </c>
       <c r="N409" s="4" t="n">
         <v>5.13</v>
@@ -42650,10 +42650,10 @@
         <v>0</v>
       </c>
       <c r="AB409" s="4" t="n">
-        <v>40.28</v>
+        <v>40.27</v>
       </c>
       <c r="AC409" s="4" t="n">
-        <v>59.72</v>
+        <v>59.73</v>
       </c>
       <c r="AD409" s="4" t="n">
         <v>0</v>
@@ -42701,7 +42701,7 @@
         </is>
       </c>
       <c r="I410" s="4" t="n">
-        <v>-41.39</v>
+        <v>-41.4</v>
       </c>
       <c r="J410" s="4" t="n">
         <v>0</v>
@@ -42721,7 +42721,7 @@
         <v>5.13</v>
       </c>
       <c r="O410" s="4" t="n">
-        <v>-41.39</v>
+        <v>-41.4</v>
       </c>
       <c r="P410" s="4" t="n">
         <v>-2.49</v>
@@ -42803,7 +42803,7 @@
         </is>
       </c>
       <c r="I411" s="4" t="n">
-        <v>-20.32</v>
+        <v>-20.33</v>
       </c>
       <c r="J411" s="4" t="n">
         <v>0.2</v>
@@ -42823,7 +42823,7 @@
         <v>5.13</v>
       </c>
       <c r="O411" s="4" t="n">
-        <v>-20.32</v>
+        <v>-20.33</v>
       </c>
       <c r="P411" s="4" t="n">
         <v>-1.89</v>
@@ -42905,7 +42905,7 @@
         </is>
       </c>
       <c r="I412" s="4" t="n">
-        <v>-2.56</v>
+        <v>-2.57</v>
       </c>
       <c r="J412" s="4" t="n">
         <v>28.2</v>
@@ -42925,7 +42925,7 @@
         <v>5.13</v>
       </c>
       <c r="O412" s="4" t="n">
-        <v>-2.25</v>
+        <v>-2.26</v>
       </c>
       <c r="P412" s="4" t="n">
         <v>-0.33</v>
@@ -43027,7 +43027,7 @@
         </is>
       </c>
       <c r="M413" s="4" t="n">
-        <v>26.25</v>
+        <v>26.24</v>
       </c>
       <c r="N413" s="4" t="n">
         <v>5.13</v>
@@ -43115,7 +43115,7 @@
         </is>
       </c>
       <c r="I414" s="4" t="n">
-        <v>-15.51</v>
+        <v>-15.52</v>
       </c>
       <c r="J414" s="4" t="n">
         <v>0.6</v>
@@ -43129,13 +43129,13 @@
         </is>
       </c>
       <c r="M414" s="4" t="n">
-        <v>-16.88</v>
+        <v>-16.89</v>
       </c>
       <c r="N414" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O414" s="4" t="n">
-        <v>-15.51</v>
+        <v>-15.52</v>
       </c>
       <c r="P414" s="4" t="n">
         <v>0</v>
@@ -43329,7 +43329,7 @@
         </is>
       </c>
       <c r="M416" s="4" t="n">
-        <v>-47.06</v>
+        <v>-47.07</v>
       </c>
       <c r="N416" s="4" t="n">
         <v>5.13</v>
@@ -43417,7 +43417,7 @@
         </is>
       </c>
       <c r="I417" s="4" t="n">
-        <v>48.56</v>
+        <v>48.55</v>
       </c>
       <c r="J417" s="4" t="n">
         <v>100</v>
@@ -43431,13 +43431,13 @@
         </is>
       </c>
       <c r="M417" s="4" t="n">
-        <v>36.09</v>
+        <v>36.08</v>
       </c>
       <c r="N417" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O417" s="4" t="n">
-        <v>48.56</v>
+        <v>48.55</v>
       </c>
       <c r="P417" s="4" t="n">
         <v>1.31</v>
@@ -43613,7 +43613,7 @@
         </is>
       </c>
       <c r="I419" s="4" t="n">
-        <v>-13.71</v>
+        <v>-13.72</v>
       </c>
       <c r="J419" s="4" t="n">
         <v>0.8</v>
@@ -43633,7 +43633,7 @@
         <v>5.13</v>
       </c>
       <c r="O419" s="4" t="n">
-        <v>-13.71</v>
+        <v>-13.72</v>
       </c>
       <c r="P419" s="4" t="n">
         <v>-0.8100000000000001</v>
@@ -43711,7 +43711,7 @@
         </is>
       </c>
       <c r="I420" s="4" t="n">
-        <v>-3.05</v>
+        <v>-3.06</v>
       </c>
       <c r="J420" s="4" t="n">
         <v>26.3</v>
@@ -43819,7 +43819,7 @@
         </is>
       </c>
       <c r="I421" s="4" t="n">
-        <v>-11.64</v>
+        <v>-11.65</v>
       </c>
       <c r="J421" s="4" t="n">
         <v>1.2</v>
@@ -43833,13 +43833,13 @@
         </is>
       </c>
       <c r="M421" s="4" t="n">
-        <v>-12.3</v>
+        <v>-12.31</v>
       </c>
       <c r="N421" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O421" s="4" t="n">
-        <v>-11.64</v>
+        <v>-11.65</v>
       </c>
       <c r="P421" s="4" t="n">
         <v>0</v>
@@ -43935,7 +43935,7 @@
         </is>
       </c>
       <c r="M422" s="4" t="n">
-        <v>-18.53</v>
+        <v>-18.54</v>
       </c>
       <c r="N422" s="4" t="n">
         <v>5.13</v>
@@ -43972,10 +43972,10 @@
         <v>0</v>
       </c>
       <c r="AB422" s="4" t="n">
-        <v>42.71</v>
+        <v>42.7</v>
       </c>
       <c r="AC422" s="4" t="n">
-        <v>57.29</v>
+        <v>57.3</v>
       </c>
       <c r="AD422" s="4" t="n">
         <v>0</v>
@@ -44023,7 +44023,7 @@
         </is>
       </c>
       <c r="I423" s="4" t="n">
-        <v>-23.32</v>
+        <v>-23.33</v>
       </c>
       <c r="J423" s="4" t="n">
         <v>0.1</v>
@@ -44037,13 +44037,13 @@
         </is>
       </c>
       <c r="M423" s="4" t="n">
-        <v>-19.65</v>
+        <v>-19.66</v>
       </c>
       <c r="N423" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O423" s="4" t="n">
-        <v>-23.32</v>
+        <v>-23.33</v>
       </c>
       <c r="P423" s="4" t="n">
         <v>-3.11</v>
@@ -44125,7 +44125,7 @@
         </is>
       </c>
       <c r="I424" s="4" t="n">
-        <v>-14.59</v>
+        <v>-14.6</v>
       </c>
       <c r="J424" s="4" t="n">
         <v>0.7</v>
@@ -44145,7 +44145,7 @@
         <v>5.13</v>
       </c>
       <c r="O424" s="4" t="n">
-        <v>-14.59</v>
+        <v>-14.6</v>
       </c>
       <c r="P424" s="4" t="n">
         <v>-1.33</v>
@@ -44227,13 +44227,13 @@
         </is>
       </c>
       <c r="I425" s="4" t="n">
-        <v>10.99</v>
+        <v>11.13</v>
       </c>
       <c r="J425" s="4" t="n">
-        <v>98.09999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K425" s="4" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="L425" t="inlineStr">
         <is>
@@ -44284,10 +44284,10 @@
         <v>0</v>
       </c>
       <c r="AB425" s="4" t="n">
-        <v>55.5</v>
+        <v>55.56</v>
       </c>
       <c r="AC425" s="4" t="n">
-        <v>44.5</v>
+        <v>44.44</v>
       </c>
       <c r="AD425" s="4" t="n">
         <v>0</v>
@@ -44335,7 +44335,7 @@
         </is>
       </c>
       <c r="I426" s="4" t="n">
-        <v>53.35</v>
+        <v>53.34</v>
       </c>
       <c r="J426" s="4" t="n">
         <v>100</v>
@@ -44349,13 +44349,13 @@
         </is>
       </c>
       <c r="M426" s="4" t="n">
-        <v>38.61</v>
+        <v>38.6</v>
       </c>
       <c r="N426" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O426" s="4" t="n">
-        <v>53.35</v>
+        <v>53.34</v>
       </c>
       <c r="P426" s="4" t="n">
         <v>0</v>
@@ -44433,7 +44433,7 @@
         </is>
       </c>
       <c r="I427" s="4" t="n">
-        <v>60.97</v>
+        <v>60.96</v>
       </c>
       <c r="J427" s="4" t="n">
         <v>100</v>
@@ -44447,13 +44447,13 @@
         </is>
       </c>
       <c r="M427" s="4" t="n">
-        <v>54.32</v>
+        <v>54.31</v>
       </c>
       <c r="N427" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O427" s="4" t="n">
-        <v>60.97</v>
+        <v>60.96</v>
       </c>
       <c r="P427" s="4" t="n">
         <v>0.21</v>
@@ -44549,13 +44549,13 @@
         </is>
       </c>
       <c r="M428" s="4" t="n">
-        <v>-17.81</v>
+        <v>-17.82</v>
       </c>
       <c r="N428" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O428" s="4" t="n">
-        <v>-18.88</v>
+        <v>-18.89</v>
       </c>
       <c r="P428" s="4" t="n">
         <v>-1.61</v>
@@ -44633,7 +44633,7 @@
         </is>
       </c>
       <c r="I429" s="4" t="n">
-        <v>-9.19</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="J429" s="4" t="n">
         <v>6.2</v>
@@ -44653,7 +44653,7 @@
         <v>5.13</v>
       </c>
       <c r="O429" s="4" t="n">
-        <v>-9.19</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="P429" s="4" t="n">
         <v>-1.93</v>
@@ -44731,7 +44731,7 @@
         </is>
       </c>
       <c r="I430" s="4" t="n">
-        <v>45.44</v>
+        <v>45.43</v>
       </c>
       <c r="J430" s="4" t="n">
         <v>100</v>
@@ -44751,7 +44751,7 @@
         <v>5.13</v>
       </c>
       <c r="O430" s="4" t="n">
-        <v>45.44</v>
+        <v>45.43</v>
       </c>
       <c r="P430" s="4" t="n">
         <v>0</v>
@@ -44833,7 +44833,7 @@
         </is>
       </c>
       <c r="I431" s="4" t="n">
-        <v>7.64</v>
+        <v>7.66</v>
       </c>
       <c r="J431" s="4" t="n">
         <v>89.5</v>
@@ -44853,7 +44853,7 @@
         <v>5.13</v>
       </c>
       <c r="O431" s="4" t="n">
-        <v>10.53</v>
+        <v>10.52</v>
       </c>
       <c r="P431" s="4" t="n">
         <v>0.16</v>
@@ -44890,10 +44890,10 @@
         <v>0</v>
       </c>
       <c r="AB431" s="4" t="n">
-        <v>53.82</v>
+        <v>53.83</v>
       </c>
       <c r="AC431" s="4" t="n">
-        <v>46.18</v>
+        <v>46.17</v>
       </c>
       <c r="AD431" s="4" t="n">
         <v>0</v>
@@ -44940,10 +44940,10 @@
         <v>2.52</v>
       </c>
       <c r="J432" s="4" t="n">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="K432" s="4" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="L432" t="inlineStr">
         <is>
@@ -44951,7 +44951,7 @@
         </is>
       </c>
       <c r="M432" s="4" t="n">
-        <v>-4.57</v>
+        <v>-4.58</v>
       </c>
       <c r="N432" s="4" t="n">
         <v>5.13</v>
@@ -45090,10 +45090,10 @@
         <v>0</v>
       </c>
       <c r="AB433" s="4" t="n">
-        <v>41.68</v>
+        <v>41.67</v>
       </c>
       <c r="AC433" s="4" t="n">
-        <v>58.32</v>
+        <v>58.33</v>
       </c>
       <c r="AD433" s="4" t="n">
         <v>0</v>
@@ -45259,7 +45259,7 @@
         <v>5.13</v>
       </c>
       <c r="O435" s="4" t="n">
-        <v>-14.18</v>
+        <v>-14.19</v>
       </c>
       <c r="P435" s="4" t="n">
         <v>-2.01</v>
@@ -45290,10 +45290,10 @@
         <v>0</v>
       </c>
       <c r="AB435" s="4" t="n">
-        <v>41.71</v>
+        <v>41.7</v>
       </c>
       <c r="AC435" s="4" t="n">
-        <v>56.11</v>
+        <v>56.12</v>
       </c>
       <c r="AD435" s="4" t="n">
         <v>2.18</v>
@@ -45853,13 +45853,13 @@
         </is>
       </c>
       <c r="I441" s="4" t="n">
-        <v>1.53</v>
+        <v>1.61</v>
       </c>
       <c r="J441" s="4" t="n">
-        <v>67.8</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K441" s="4" t="n">
-        <v>32.2</v>
+        <v>31.9</v>
       </c>
       <c r="L441" t="inlineStr">
         <is>
@@ -45910,10 +45910,10 @@
         <v>0</v>
       </c>
       <c r="AB441" s="4" t="n">
-        <v>50.77</v>
+        <v>50.8</v>
       </c>
       <c r="AC441" s="4" t="n">
-        <v>49.23</v>
+        <v>49.2</v>
       </c>
       <c r="AD441" s="4" t="n">
         <v>0</v>
@@ -46879,7 +46879,7 @@
         </is>
       </c>
       <c r="I451" s="4" t="n">
-        <v>36.3</v>
+        <v>36.29</v>
       </c>
       <c r="J451" s="4" t="n">
         <v>100</v>
@@ -46893,13 +46893,13 @@
         </is>
       </c>
       <c r="M451" s="4" t="n">
-        <v>20.6</v>
+        <v>20.58</v>
       </c>
       <c r="N451" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O451" s="4" t="n">
-        <v>36.32</v>
+        <v>36.29</v>
       </c>
       <c r="P451" s="4" t="n">
         <v>1.82</v>
@@ -47191,13 +47191,13 @@
         </is>
       </c>
       <c r="I454" s="4" t="n">
-        <v>5.09</v>
+        <v>5.14</v>
       </c>
       <c r="J454" s="4" t="n">
-        <v>81.2</v>
+        <v>81.3</v>
       </c>
       <c r="K454" s="4" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L454" t="inlineStr">
         <is>
@@ -47248,10 +47248,10 @@
         <v>0</v>
       </c>
       <c r="AB454" s="4" t="n">
-        <v>52.54</v>
+        <v>52.57</v>
       </c>
       <c r="AC454" s="4" t="n">
-        <v>47.46</v>
+        <v>47.43</v>
       </c>
       <c r="AD454" s="4" t="n">
         <v>0</v>
@@ -47397,7 +47397,7 @@
         </is>
       </c>
       <c r="I456" s="4" t="n">
-        <v>-22.74</v>
+        <v>-22.8</v>
       </c>
       <c r="J456" s="4" t="n">
         <v>0.1</v>
@@ -47454,10 +47454,10 @@
         <v>0</v>
       </c>
       <c r="AB456" s="4" t="n">
-        <v>38.63</v>
+        <v>38.6</v>
       </c>
       <c r="AC456" s="4" t="n">
-        <v>61.37</v>
+        <v>61.4</v>
       </c>
       <c r="AD456" s="4" t="n">
         <v>0</v>
@@ -48137,7 +48137,7 @@
         </is>
       </c>
       <c r="M463" s="4" t="n">
-        <v>41.85</v>
+        <v>41.86</v>
       </c>
       <c r="N463" s="4" t="n">
         <v>5.13</v>
@@ -48225,13 +48225,13 @@
         </is>
       </c>
       <c r="I464" s="4" t="n">
-        <v>3.69</v>
+        <v>3.71</v>
       </c>
       <c r="J464" s="4" t="n">
-        <v>76.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="K464" s="4" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="L464" t="inlineStr">
         <is>
@@ -48282,10 +48282,10 @@
         <v>0</v>
       </c>
       <c r="AB464" s="4" t="n">
-        <v>51.85</v>
+        <v>51.86</v>
       </c>
       <c r="AC464" s="4" t="n">
-        <v>48.15</v>
+        <v>48.14</v>
       </c>
       <c r="AD464" s="4" t="n">
         <v>0</v>
@@ -48333,7 +48333,7 @@
         </is>
       </c>
       <c r="I465" s="4" t="n">
-        <v>62.34</v>
+        <v>62.35</v>
       </c>
       <c r="J465" s="4" t="n">
         <v>100</v>
@@ -48353,7 +48353,7 @@
         <v>5.13</v>
       </c>
       <c r="O465" s="4" t="n">
-        <v>62.34</v>
+        <v>62.35</v>
       </c>
       <c r="P465" s="4" t="n">
         <v>0</v>
@@ -48449,7 +48449,7 @@
         </is>
       </c>
       <c r="M466" s="4" t="n">
-        <v>-22.2</v>
+        <v>-22.19</v>
       </c>
       <c r="N466" s="4" t="n">
         <v>5.13</v>
@@ -48486,10 +48486,10 @@
         <v>0</v>
       </c>
       <c r="AB466" s="4" t="n">
-        <v>37.59</v>
+        <v>37.6</v>
       </c>
       <c r="AC466" s="4" t="n">
-        <v>62.41</v>
+        <v>62.4</v>
       </c>
       <c r="AD466" s="4" t="n">
         <v>0</v>
@@ -48537,7 +48537,7 @@
         </is>
       </c>
       <c r="I467" s="4" t="n">
-        <v>-18.94</v>
+        <v>-18.93</v>
       </c>
       <c r="J467" s="4" t="n">
         <v>0.3</v>
@@ -48551,13 +48551,13 @@
         </is>
       </c>
       <c r="M467" s="4" t="n">
-        <v>-15.81</v>
+        <v>-15.8</v>
       </c>
       <c r="N467" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O467" s="4" t="n">
-        <v>-18.03</v>
+        <v>-18.02</v>
       </c>
       <c r="P467" s="4" t="n">
         <v>-1.71</v>
@@ -48594,10 +48594,10 @@
         <v>0</v>
       </c>
       <c r="AB467" s="4" t="n">
-        <v>40.53</v>
+        <v>40.54</v>
       </c>
       <c r="AC467" s="4" t="n">
-        <v>59.47</v>
+        <v>59.46</v>
       </c>
       <c r="AD467" s="4" t="n">
         <v>0</v>
@@ -48641,7 +48641,7 @@
         </is>
       </c>
       <c r="I468" s="4" t="n">
-        <v>-18.83</v>
+        <v>-18.82</v>
       </c>
       <c r="J468" s="4" t="n">
         <v>0.3</v>
@@ -48655,13 +48655,13 @@
         </is>
       </c>
       <c r="M468" s="4" t="n">
-        <v>-21.43</v>
+        <v>-21.42</v>
       </c>
       <c r="N468" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O468" s="4" t="n">
-        <v>-18.83</v>
+        <v>-18.82</v>
       </c>
       <c r="P468" s="4" t="n">
         <v>-1.54</v>
@@ -48794,10 +48794,10 @@
         <v>0</v>
       </c>
       <c r="AB469" s="4" t="n">
-        <v>42.77</v>
+        <v>42.78</v>
       </c>
       <c r="AC469" s="4" t="n">
-        <v>57.23</v>
+        <v>57.22</v>
       </c>
       <c r="AD469" s="4" t="n">
         <v>0</v>
@@ -49147,13 +49147,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-1.2</v>
+        <v>-0.91</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>46.8</v>
+        <v>47.3</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>53.2</v>
+        <v>52.7</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49161,13 +49161,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.72</v>
+        <v>-10.54</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.17</v>
+        <v>-1.99</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.37</v>
@@ -49204,10 +49204,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.37</v>
+        <v>45.42</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.63</v>
+        <v>46.58</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -49722,10 +49722,10 @@
         <v>0</v>
       </c>
       <c r="AB478" s="4" t="n">
-        <v>47.2</v>
+        <v>47.21</v>
       </c>
       <c r="AC478" s="4" t="n">
-        <v>52.8</v>
+        <v>52.79</v>
       </c>
       <c r="AD478" s="4" t="n">
         <v>0</v>
@@ -49787,13 +49787,13 @@
         </is>
       </c>
       <c r="M479" s="4" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="N479" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O479" s="4" t="n">
-        <v>12.88</v>
+        <v>12.87</v>
       </c>
       <c r="P479" s="4" t="n">
         <v>1.71</v>
@@ -49877,13 +49877,13 @@
         </is>
       </c>
       <c r="I480" s="4" t="n">
-        <v>-1.49</v>
+        <v>-1.5</v>
       </c>
       <c r="J480" s="4" t="n">
-        <v>32.4</v>
+        <v>32.3</v>
       </c>
       <c r="K480" s="4" t="n">
-        <v>67.59999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="L480" t="inlineStr">
         <is>
@@ -49985,7 +49985,7 @@
         </is>
       </c>
       <c r="I481" s="4" t="n">
-        <v>-39.35</v>
+        <v>-39.36</v>
       </c>
       <c r="J481" s="4" t="n">
         <v>0</v>
@@ -50505,7 +50505,7 @@
         </is>
       </c>
       <c r="I486" s="4" t="n">
-        <v>29.78</v>
+        <v>29.81</v>
       </c>
       <c r="J486" s="4" t="n">
         <v>100</v>
@@ -50525,7 +50525,7 @@
         <v>5.13</v>
       </c>
       <c r="O486" s="4" t="n">
-        <v>35.74</v>
+        <v>35.75</v>
       </c>
       <c r="P486" s="4" t="n">
         <v>0.66</v>
@@ -50562,10 +50562,10 @@
         <v>0</v>
       </c>
       <c r="AB486" s="4" t="n">
-        <v>64.89</v>
+        <v>64.91</v>
       </c>
       <c r="AC486" s="4" t="n">
-        <v>35.11</v>
+        <v>35.09</v>
       </c>
       <c r="AD486" s="4" t="n">
         <v>0</v>
@@ -50613,13 +50613,13 @@
         </is>
       </c>
       <c r="I487" s="4" t="n">
-        <v>2.12</v>
+        <v>2.09</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>70.09999999999999</v>
+        <v>70</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>29.9</v>
+        <v>30</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -50627,7 +50627,7 @@
         </is>
       </c>
       <c r="M487" s="4" t="n">
-        <v>8.74</v>
+        <v>8.73</v>
       </c>
       <c r="N487" s="4" t="n">
         <v>5.13</v>
@@ -50670,10 +50670,10 @@
         <v>0</v>
       </c>
       <c r="AB487" s="4" t="n">
-        <v>51.06</v>
+        <v>51.04</v>
       </c>
       <c r="AC487" s="4" t="n">
-        <v>48.94</v>
+        <v>48.96</v>
       </c>
       <c r="AD487" s="4" t="n">
         <v>0</v>
@@ -50717,7 +50717,7 @@
         </is>
       </c>
       <c r="I488" s="4" t="n">
-        <v>5.04</v>
+        <v>5.05</v>
       </c>
       <c r="J488" s="4" t="n">
         <v>81</v>
@@ -50774,10 +50774,10 @@
         <v>0</v>
       </c>
       <c r="AB488" s="4" t="n">
-        <v>52.52</v>
+        <v>52.53</v>
       </c>
       <c r="AC488" s="4" t="n">
-        <v>47.48</v>
+        <v>47.47</v>
       </c>
       <c r="AD488" s="4" t="n">
         <v>0</v>
@@ -50835,7 +50835,7 @@
         </is>
       </c>
       <c r="M489" s="4" t="n">
-        <v>6.87</v>
+        <v>6.86</v>
       </c>
       <c r="N489" s="4" t="n">
         <v>5.13</v>
@@ -51037,7 +51037,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-20.82</v>
+        <v>-21</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>4.9</v>
@@ -51092,16 +51092,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>9.710000000000001</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>32.91</v>
+        <v>32.73</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.72</v>
+        <v>53.74</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51253,13 +51253,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-6.51</v>
+        <v>-6.95</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>30.5</v>
+        <v>29.2</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>69.5</v>
+        <v>70.8</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51308,16 +51308,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>46.74</v>
+        <v>46.52</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>30.5</v>
+        <v>29.2</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>53.26</v>
+        <v>53.48</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>
@@ -51361,7 +51361,7 @@
         </is>
       </c>
       <c r="I494" s="4" t="n">
-        <v>7.1</v>
+        <v>7.11</v>
       </c>
       <c r="J494" s="4" t="n">
         <v>87.8</v>
@@ -51375,7 +51375,7 @@
         </is>
       </c>
       <c r="M494" s="4" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="N494" s="4" t="n">
         <v>5.13</v>
@@ -51571,7 +51571,7 @@
         </is>
       </c>
       <c r="I496" s="4" t="n">
-        <v>18.61</v>
+        <v>18.62</v>
       </c>
       <c r="J496" s="4" t="n">
         <v>99.7</v>
@@ -51585,13 +51585,13 @@
         </is>
       </c>
       <c r="M496" s="4" t="n">
-        <v>7.53</v>
+        <v>7.54</v>
       </c>
       <c r="N496" s="4" t="n">
         <v>5.13</v>
       </c>
       <c r="O496" s="4" t="n">
-        <v>18.61</v>
+        <v>18.62</v>
       </c>
       <c r="P496" s="4" t="n">
         <v>3.16</v>
@@ -51693,7 +51693,7 @@
         <v>5.13</v>
       </c>
       <c r="O497" s="4" t="n">
-        <v>-1.95</v>
+        <v>-1.96</v>
       </c>
       <c r="P497" s="4" t="n">
         <v>0.6</v>
@@ -51893,7 +51893,7 @@
         </is>
       </c>
       <c r="M499" s="4" t="n">
-        <v>12.55</v>
+        <v>12.56</v>
       </c>
       <c r="N499" s="4" t="n">
         <v>5.13</v>
@@ -51981,7 +51981,7 @@
         </is>
       </c>
       <c r="I500" s="4" t="n">
-        <v>22.77</v>
+        <v>22.82</v>
       </c>
       <c r="J500" s="4" t="n">
         <v>99.90000000000001</v>
@@ -51995,7 +51995,7 @@
         </is>
       </c>
       <c r="M500" s="4" t="n">
-        <v>17.1</v>
+        <v>17.11</v>
       </c>
       <c r="N500" s="4" t="n">
         <v>5.13</v>
@@ -52038,10 +52038,10 @@
         <v>0</v>
       </c>
       <c r="AB500" s="4" t="n">
-        <v>61.39</v>
+        <v>61.41</v>
       </c>
       <c r="AC500" s="4" t="n">
-        <v>38.61</v>
+        <v>38.59</v>
       </c>
       <c r="AD500" s="4" t="n">
         <v>0</v>
@@ -52397,7 +52397,7 @@
         </is>
       </c>
       <c r="I504" s="4" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="J504" s="4" t="n">
         <v>63.2</v>
@@ -52933,7 +52933,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -53627,7 +53627,7 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>121.4</v>
+        <v>121.5</v>
       </c>
       <c r="K14" t="n">
         <v>125</v>
@@ -55089,7 +55089,7 @@
         <v>112</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>72.8</v>
+        <v>72.7</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -55547,13 +55547,13 @@
         <v>42</v>
       </c>
       <c r="L47" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M47" t="n">
         <v>53</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TX-32: correct Dem nominee to Dan Barrios
Alex Cornwallis (C-0925) was carried as the *projected* Dem nominee, but
Dan Barrios won the March 3 primary. Add C-1046 Dan Barrios and repoint
TX-32; dem_status projected -> confirmed. C-0925 is left in place as an
orphan, matching the 19 existing primary-loser rows.

Strength stays 0.0 (same as Cornwallis), so TX-32's forecast is unchanged
at D 18.2% / Likely R -- this is a name/id/status correction only.

Reran 2026-07-28 + 2026-07-29. Movement in the 12 AK/ME/MT/NE RCV and
three-way races is unseeded Monte-Carlo noise from the rerun, not signal.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>49.4</v>
+        <v>50.5</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.2</v>
+        <v>232.1</v>
       </c>
       <c r="C9" t="n">
-        <v>202.8</v>
+        <v>202.9</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>80.90000000000001</v>
+        <v>80.2</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>40.3</v>
+        <v>40.6</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-2.96</v>
+        <v>-3.29</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>39.8</v>
+        <v>40.9</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>60.2</v>
+        <v>59.1</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4695,13 +4695,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.95</v>
+        <v>-2.98</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>42</v>
+        <v>40.1</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>58</v>
+        <v>59.9</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4709,13 +4709,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.49</v>
+        <v>-2.54</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.15</v>
+        <v>-1.2</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.1</v>
@@ -4750,16 +4750,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.53</v>
+        <v>48.51</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>42</v>
+        <v>40.1</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.47</v>
+        <v>51.49</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -24673,7 +24673,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>31.04</v>
+        <v>30.56</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24771,13 +24771,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.14</v>
+        <v>-4.31</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>36.4</v>
+        <v>35.3</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>63.6</v>
+        <v>64.7</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28261,7 +28261,7 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.26</v>
+        <v>-6.24</v>
       </c>
       <c r="J269" s="4" t="n">
         <v>14.9</v>
@@ -28275,13 +28275,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-11.51</v>
+        <v>-11.49</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-7.47</v>
+        <v>-7.45</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28318,10 +28318,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.87</v>
+        <v>46.88</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.13</v>
+        <v>53.12</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28369,7 +28369,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.21</v>
+        <v>-33.18</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28383,13 +28383,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-30.48</v>
+        <v>-30.45</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.21</v>
+        <v>-33.18</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28420,10 +28420,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.4</v>
+        <v>33.41</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>66.59</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -30025,13 +30025,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.699999999999999</v>
+        <v>-9.67</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>95.09999999999999</v>
+        <v>95</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -30039,13 +30039,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.970000000000001</v>
+        <v>-8.93</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-10.29</v>
+        <v>-10.25</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30082,10 +30082,10 @@
         <v>0</v>
       </c>
       <c r="AB286" s="4" t="n">
-        <v>45.15</v>
+        <v>45.17</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>54.85</v>
+        <v>54.83</v>
       </c>
       <c r="AD286" s="4" t="n">
         <v>0</v>
@@ -30129,7 +30129,7 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>12.46</v>
+        <v>12.49</v>
       </c>
       <c r="J287" s="4" t="n">
         <v>98.90000000000001</v>
@@ -30143,13 +30143,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>8.890000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.13</v>
+        <v>14.17</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30186,10 +30186,10 @@
         <v>0</v>
       </c>
       <c r="AB287" s="4" t="n">
-        <v>56.23</v>
+        <v>56.25</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>43.77</v>
+        <v>43.75</v>
       </c>
       <c r="AD287" s="4" t="n">
         <v>0</v>
@@ -30237,7 +30237,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.84</v>
+        <v>-52.8</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30251,13 +30251,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.92</v>
+        <v>-49.88</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.84</v>
+        <v>-52.8</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30288,10 +30288,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.58</v>
+        <v>23.6</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.42</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -44624,7 +44624,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Alex Cornwallis</t>
+          <t>Dan Barrios</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
@@ -49153,13 +49153,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.72</v>
+        <v>-0.66</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>47.4</v>
+        <v>47.8</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>52.6</v>
+        <v>52.2</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49167,13 +49167,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.56</v>
+        <v>-10.65</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-1.97</v>
+        <v>-2.06</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.37</v>
@@ -49210,10 +49210,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.42</v>
+        <v>45.39</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.58</v>
+        <v>46.61</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -51043,13 +51043,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-22.79</v>
+        <v>-22.7</v>
       </c>
       <c r="J491" s="4" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>96.40000000000001</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51098,16 +51098,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>11.63</v>
+        <v>11.66</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>30.96</v>
+        <v>30.99</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.75</v>
+        <v>53.69</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51259,13 +51259,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-6.69</v>
+        <v>-6.48</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>30.1</v>
+        <v>31.6</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>69.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51314,16 +51314,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>46.65</v>
+        <v>46.76</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>30.1</v>
+        <v>31.6</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>53.35</v>
+        <v>53.24</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
OH-07 de-spoilered strength + LA-06 open (Fields out); rerun 2026-07-29
Max Miller's candidate strength -4.37 -> -0.5. The inherited value credited him
with a personal R+4.4 that was an artifact of 2024's three-way race (Kucinich,
a former Dem congressman, took 12.8% out of the Dem column). Netting the spoiler
out (2/3 D / 1/3 R) puts Miller at par with the district's R+11.1 pres lean;
2022's clean two-way puts him ~1 pt off par. OH-07: -7.6 -> -5.4, Likely R ->
Lean R.

Cleo Fields dropped from LA-06 (announced 2026-07-21 he won't seek reelection
after the post-Callais map redrew the seat R+32; running for state Senate D14).
Dem slot -> placeholder C-1047, incumbent_party cleared (seat_holder stays DEM),
C-0499 incumbent flag 0, LA-06 candidate_meta row removed. LA-06: -20.1 -> -28.1.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="C8" t="n">
-        <v>49.5</v>
+        <v>49.4</v>
       </c>
       <c r="D8" t="n">
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>50.5</v>
+        <v>50.9</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -575,7 +575,7 @@
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>80.2</v>
+        <v>80.8</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="C10" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="D10" t="n">
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>40.6</v>
+        <v>40.1</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.29</v>
+        <v>-3.35</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>40.9</v>
+        <v>39.9</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>59.1</v>
+        <v>60.1</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Toss-up</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4695,13 +4695,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.98</v>
+        <v>-3.04</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>40.1</v>
+        <v>40.6</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>59.9</v>
+        <v>59.4</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4709,13 +4709,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.54</v>
+        <v>-2.61</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.2</v>
+        <v>-1.27</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.1</v>
@@ -4750,16 +4750,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.51</v>
+        <v>48.48</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>40.1</v>
+        <v>40.6</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.49</v>
+        <v>51.52</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -22830,7 +22830,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Cleo Fields</t>
+          <t>Democratic candidate (LA-06)</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -22838,24 +22838,20 @@
           <t>Peter Williams</t>
         </is>
       </c>
-      <c r="G216" t="inlineStr">
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>DEM</t>
-        </is>
-      </c>
       <c r="I216" s="4" t="n">
-        <v>-20.11</v>
+        <v>-28.11</v>
       </c>
       <c r="J216" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K216" s="4" t="n">
-        <v>99.8</v>
+        <v>100</v>
       </c>
       <c r="L216" t="inlineStr">
         <is>
@@ -22869,13 +22865,13 @@
         <v>5.17</v>
       </c>
       <c r="O216" s="4" t="n">
-        <v>-20.11</v>
+        <v>-28.11</v>
       </c>
       <c r="P216" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q216" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R216" s="4" t="n">
         <v>-32.4</v>
@@ -22900,10 +22896,10 @@
         <v>0</v>
       </c>
       <c r="AB216" s="4" t="n">
-        <v>39.95</v>
+        <v>35.95</v>
       </c>
       <c r="AC216" s="4" t="n">
-        <v>60.05</v>
+        <v>64.05</v>
       </c>
       <c r="AD216" s="4" t="n">
         <v>0</v>
@@ -24673,7 +24669,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.56</v>
+        <v>30.48</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24771,13 +24767,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.31</v>
+        <v>-4.97</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>35.3</v>
+        <v>34.6</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>64.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28261,13 +28257,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.24</v>
+        <v>-6.29</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>85.09999999999999</v>
+        <v>85.2</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28275,13 +28271,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-11.49</v>
+        <v>-11.56</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-7.45</v>
+        <v>-7.52</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28318,10 +28314,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.88</v>
+        <v>46.86</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.12</v>
+        <v>53.14</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28369,7 +28365,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.18</v>
+        <v>-33.25</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28383,13 +28379,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-30.45</v>
+        <v>-30.52</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.18</v>
+        <v>-33.25</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28420,10 +28416,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.41</v>
+        <v>33.37</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.59</v>
+        <v>66.63</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -30025,7 +30021,7 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.67</v>
+        <v>-9.65</v>
       </c>
       <c r="J286" s="4" t="n">
         <v>5</v>
@@ -30035,17 +30031,17 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>Safe R</t>
+          <t>Likely R</t>
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.93</v>
+        <v>-8.91</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-10.25</v>
+        <v>-10.24</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30129,7 +30125,7 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>12.49</v>
+        <v>12.51</v>
       </c>
       <c r="J287" s="4" t="n">
         <v>98.90000000000001</v>
@@ -30143,13 +30139,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>8.93</v>
+        <v>8.94</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.17</v>
+        <v>14.18</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30237,7 +30233,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.8</v>
+        <v>-52.78</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30251,13 +30247,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.88</v>
+        <v>-49.87</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.8</v>
+        <v>-52.78</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30288,10 +30284,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.6</v>
+        <v>23.61</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.40000000000001</v>
+        <v>76.39</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -35773,13 +35769,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>-6.66</v>
+        <v>-4.86</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>13.6</v>
+        <v>19.6</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>86.40000000000001</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35793,13 +35789,13 @@
         <v>5.17</v>
       </c>
       <c r="O342" s="4" t="n">
-        <v>-7.82</v>
+        <v>-5.24</v>
       </c>
       <c r="P342" s="4" t="n">
         <v>-0.51</v>
       </c>
       <c r="Q342" s="4" t="n">
-        <v>-4.58</v>
+        <v>-2</v>
       </c>
       <c r="R342" s="4" t="n">
         <v>-11.15</v>
@@ -35830,10 +35826,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>46.67</v>
+        <v>47.57</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>53.33</v>
+        <v>52.43</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -49153,13 +49149,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.66</v>
+        <v>-0.95</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>47.8</v>
+        <v>47.6</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>52.2</v>
+        <v>52.4</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49167,13 +49163,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.65</v>
+        <v>-10.66</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.17</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.06</v>
+        <v>-2.07</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.37</v>
@@ -51043,13 +51039,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-22.7</v>
+        <v>-22.98</v>
       </c>
       <c r="J491" s="4" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>96.59999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51098,16 +51094,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>11.66</v>
+        <v>11.21</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>30.99</v>
+        <v>31.08</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.69</v>
+        <v>54.06</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51259,13 +51255,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-6.48</v>
+        <v>-6.41</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>31.6</v>
+        <v>30.8</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>68.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51314,16 +51310,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>46.76</v>
+        <v>46.79</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>31.6</v>
+        <v>30.8</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>53.24</v>
+        <v>53.21</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>
@@ -52939,7 +52935,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -55550,7 +55546,7 @@
         <v>41</v>
       </c>
       <c r="K47" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L47" t="n">
         <v>27</v>

</xml_diff>

<commit_message>
Forecast 2026-08-07: SD-GOV Rhoden, TN primary nominees
SD-GOV: Doeden led the June 2 primary but cleared no 35% threshold; Rhoden
won the July 28 runoff 70.8-29.2. Rep slot back to the incumbent governor
(C-0134), status confirmed.

TN (Aug 6 primaries), all slots confirmed:
- TN-05 Ogles LOST to Charlie Hatcher 53.2-46.8 -> open seat, Safe R to Likely R
- TN-06 Johnny Garrett (R) / Mike Croley (D) for the open Rose seat
- TN-03 Anna Golladay (D), TN-08 Heidi Kuhn (D)
- TN-GOV Blackburn/Green, TN-SEN Hagerty/Bradshaw and the rest confirmed as projected

Fundraising re-scraped before the run so the changed slots stopped carrying
the old candidates' money (TN-05 rep $613k Ogles -> $719k Hatcher; TN-06 rep
$1.55M Hilleary -> $2.38M Garrett).

Dropped candidate_meta's VA-04 "Robert Murray" row: it matched Robert Murray
Morris, a cavalry officer who died in 1896.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="C8" t="n">
-        <v>49.6</v>
+        <v>49.5</v>
       </c>
       <c r="D8" t="n">
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>49</v>
+        <v>50.2</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.7</v>
+        <v>232.3</v>
       </c>
       <c r="C9" t="n">
-        <v>202.3</v>
+        <v>202.7</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>82.59999999999999</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>24</v>
       </c>
       <c r="E10" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.4</v>
+        <v>-3.18</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>39.1</v>
+        <v>40.5</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>60.9</v>
+        <v>59.5</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4067,23 +4067,27 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Toby Doeden</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>Larry Rhoden</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>REP</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>REP</t>
         </is>
       </c>
       <c r="I32" s="4" t="n">
-        <v>-25.16</v>
+        <v>-25.8</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -4097,13 +4101,13 @@
         <v>5.27</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>-25.16</v>
+        <v>-25.8</v>
       </c>
       <c r="P32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q32" s="4" t="n">
-        <v>0</v>
+        <v>-0.64</v>
       </c>
       <c r="R32" s="4" t="n">
         <v>-29.98</v>
@@ -4128,10 +4132,10 @@
         <v>0</v>
       </c>
       <c r="AB32" s="4" t="n">
-        <v>37.42</v>
+        <v>37.1</v>
       </c>
       <c r="AC32" s="4" t="n">
-        <v>62.58</v>
+        <v>62.9</v>
       </c>
       <c r="AD32" s="4" t="n">
         <v>0</v>
@@ -4701,13 +4705,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.45</v>
+        <v>-2.38</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28.6</v>
+        <v>28.9</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>71.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4715,13 +4719,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.6</v>
+        <v>-2.51</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.18</v>
+        <v>-1.09</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.13</v>
@@ -4756,16 +4760,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.77</v>
+        <v>48.81</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>28.6</v>
+        <v>28.9</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.23</v>
+        <v>51.19</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -24705,7 +24709,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.55</v>
+        <v>30.6</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24803,13 +24807,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-3.97</v>
+        <v>-3.85</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>37.4</v>
+        <v>37.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>62.6</v>
+        <v>62.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28293,7 +28297,7 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.79</v>
+        <v>-6.77</v>
       </c>
       <c r="J269" s="4" t="n">
         <v>13.2</v>
@@ -28307,13 +28311,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-12.21</v>
+        <v>-12.18</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-8.07</v>
+        <v>-8.029999999999999</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28350,10 +28354,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.6</v>
+        <v>46.62</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.4</v>
+        <v>53.38</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28401,7 +28405,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.8</v>
+        <v>-33.77</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28415,13 +28419,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-31.17</v>
+        <v>-31.14</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.8</v>
+        <v>-33.77</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28452,10 +28456,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.1</v>
+        <v>33.11</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.90000000000001</v>
+        <v>66.89</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -40521,7 +40525,7 @@
         </is>
       </c>
       <c r="I388" s="4" t="n">
-        <v>-23.56</v>
+        <v>-23.71</v>
       </c>
       <c r="J388" s="4" t="n">
         <v>0.1</v>
@@ -40535,13 +40539,13 @@
         </is>
       </c>
       <c r="M388" s="4" t="n">
-        <v>-26.61</v>
+        <v>-26.76</v>
       </c>
       <c r="N388" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O388" s="4" t="n">
-        <v>-23.56</v>
+        <v>-23.71</v>
       </c>
       <c r="P388" s="4" t="n">
         <v>-1.2</v>
@@ -40572,10 +40576,10 @@
         <v>0</v>
       </c>
       <c r="AB388" s="4" t="n">
-        <v>38.22</v>
+        <v>38.15</v>
       </c>
       <c r="AC388" s="4" t="n">
-        <v>61.78</v>
+        <v>61.85</v>
       </c>
       <c r="AD388" s="4" t="n">
         <v>0</v>
@@ -40808,7 +40812,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>Joel Hawn</t>
+          <t>Anna Golladay</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
@@ -40827,7 +40831,7 @@
         </is>
       </c>
       <c r="I391" s="4" t="n">
-        <v>-35.61</v>
+        <v>-35.05</v>
       </c>
       <c r="J391" s="4" t="n">
         <v>0</v>
@@ -40847,10 +40851,10 @@
         <v>5.27</v>
       </c>
       <c r="O391" s="4" t="n">
-        <v>-35.61</v>
+        <v>-35.05</v>
       </c>
       <c r="P391" s="4" t="n">
-        <v>-2.9</v>
+        <v>-2.34</v>
       </c>
       <c r="Q391" s="4" t="n">
         <v>-3.43</v>
@@ -40865,7 +40869,7 @@
       </c>
       <c r="V391" s="4" t="n"/>
       <c r="W391" s="5" t="n">
-        <v>140</v>
+        <v>55555</v>
       </c>
       <c r="X391" s="5" t="n">
         <v>2330803</v>
@@ -40878,10 +40882,10 @@
         <v>0</v>
       </c>
       <c r="AB391" s="4" t="n">
-        <v>32.19</v>
+        <v>32.47</v>
       </c>
       <c r="AC391" s="4" t="n">
-        <v>67.81</v>
+        <v>67.53</v>
       </c>
       <c r="AD391" s="4" t="n">
         <v>0</v>
@@ -41017,27 +41021,23 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Andy Ogles</t>
-        </is>
-      </c>
-      <c r="G393" t="inlineStr">
+          <t>Charlie Hatcher</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr">
         <is>
           <t>REP</t>
         </is>
       </c>
-      <c r="H393" t="inlineStr">
-        <is>
-          <t>REP</t>
-        </is>
-      </c>
       <c r="I393" s="4" t="n">
-        <v>-13.76</v>
+        <v>-13.11</v>
       </c>
       <c r="J393" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="K393" s="4" t="n">
-        <v>99.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="L393" t="inlineStr">
         <is>
@@ -41051,34 +41051,28 @@
         <v>5.27</v>
       </c>
       <c r="O393" s="4" t="n">
-        <v>-14.72</v>
+        <v>-13.11</v>
       </c>
       <c r="P393" s="4" t="n">
-        <v>0.87</v>
+        <v>0.96</v>
       </c>
       <c r="Q393" s="4" t="n">
-        <v>-1.53</v>
+        <v>0</v>
       </c>
       <c r="R393" s="4" t="n">
         <v>-23.39</v>
       </c>
-      <c r="S393" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="T393" s="4" t="n">
-        <v>47</v>
-      </c>
+      <c r="S393" s="4" t="n"/>
+      <c r="T393" s="4" t="n"/>
       <c r="U393" t="n">
-        <v>1</v>
-      </c>
-      <c r="V393" s="4" t="n">
-        <v>-9</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V393" s="4" t="n"/>
       <c r="W393" s="5" t="n">
         <v>2599775</v>
       </c>
       <c r="X393" s="5" t="n">
-        <v>613135</v>
+        <v>719503</v>
       </c>
       <c r="Y393" t="inlineStr"/>
       <c r="Z393" s="4" t="n">
@@ -41088,10 +41082,10 @@
         <v>0</v>
       </c>
       <c r="AB393" s="4" t="n">
-        <v>43.12</v>
+        <v>43.45</v>
       </c>
       <c r="AC393" s="4" t="n">
-        <v>56.88</v>
+        <v>56.55</v>
       </c>
       <c r="AD393" s="4" t="n">
         <v>0</v>
@@ -41120,12 +41114,12 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Chaney Mosley</t>
+          <t>Mike Croley</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Van Hilleary</t>
+          <t>Johnny Garrett</t>
         </is>
       </c>
       <c r="G394" t="inlineStr"/>
@@ -41135,7 +41129,7 @@
         </is>
       </c>
       <c r="I394" s="4" t="n">
-        <v>-20.87</v>
+        <v>-21.31</v>
       </c>
       <c r="J394" s="4" t="n">
         <v>0.2</v>
@@ -41155,10 +41149,10 @@
         <v>5.27</v>
       </c>
       <c r="O394" s="4" t="n">
-        <v>-20.87</v>
+        <v>-21.31</v>
       </c>
       <c r="P394" s="4" t="n">
-        <v>-1.63</v>
+        <v>-2.07</v>
       </c>
       <c r="Q394" s="4" t="n">
         <v>0</v>
@@ -41173,10 +41167,10 @@
       </c>
       <c r="V394" s="4" t="n"/>
       <c r="W394" s="5" t="n">
-        <v>86869</v>
+        <v>35380</v>
       </c>
       <c r="X394" s="5" t="n">
-        <v>1552429</v>
+        <v>2380327</v>
       </c>
       <c r="Y394" t="inlineStr"/>
       <c r="Z394" s="4" t="n">
@@ -41186,10 +41180,10 @@
         <v>0</v>
       </c>
       <c r="AB394" s="4" t="n">
-        <v>39.57</v>
+        <v>39.35</v>
       </c>
       <c r="AC394" s="4" t="n">
-        <v>60.43</v>
+        <v>60.65</v>
       </c>
       <c r="AD394" s="4" t="n">
         <v>0</v>
@@ -41320,7 +41314,7 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>William Wicker</t>
+          <t>Heidi Kuhn</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
@@ -41339,13 +41333,13 @@
         </is>
       </c>
       <c r="I396" s="4" t="n">
-        <v>-18.63</v>
+        <v>-21.06</v>
       </c>
       <c r="J396" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K396" s="4" t="n">
-        <v>99.7</v>
+        <v>99.8</v>
       </c>
       <c r="L396" t="inlineStr">
         <is>
@@ -41359,10 +41353,10 @@
         <v>5.27</v>
       </c>
       <c r="O396" s="4" t="n">
-        <v>-18.63</v>
+        <v>-21.06</v>
       </c>
       <c r="P396" s="4" t="n">
-        <v>0</v>
+        <v>-2.43</v>
       </c>
       <c r="Q396" s="4" t="n">
         <v>-5.48</v>
@@ -41377,7 +41371,7 @@
       </c>
       <c r="V396" s="4" t="n"/>
       <c r="W396" s="5" t="n">
-        <v>0</v>
+        <v>39805</v>
       </c>
       <c r="X396" s="5" t="n">
         <v>2232874</v>
@@ -41390,10 +41384,10 @@
         <v>0</v>
       </c>
       <c r="AB396" s="4" t="n">
-        <v>40.68</v>
+        <v>39.47</v>
       </c>
       <c r="AC396" s="4" t="n">
-        <v>59.32</v>
+        <v>60.53</v>
       </c>
       <c r="AD396" s="4" t="n">
         <v>0</v>
@@ -49193,13 +49187,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.6</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>47.6</v>
+        <v>48.5</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>52.4</v>
+        <v>51.5</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49207,13 +49201,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.67</v>
+        <v>-10.62</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.01</v>
+        <v>-1.95</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.34</v>
@@ -49250,10 +49244,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.4</v>
+        <v>45.42</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.6</v>
+        <v>46.58</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -51089,7 +51083,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-25.58</v>
+        <v>-25.45</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0.1</v>
@@ -51144,16 +51138,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>14.05</v>
+        <v>14.07</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>28.36</v>
+        <v>28.41</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.93</v>
+        <v>53.86</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -52245,7 +52239,7 @@
         </is>
       </c>
       <c r="I502" s="4" t="n">
-        <v>-20.83</v>
+        <v>-20.93</v>
       </c>
       <c r="J502" s="4" t="n">
         <v>0.2</v>
@@ -52259,13 +52253,13 @@
         </is>
       </c>
       <c r="M502" s="4" t="n">
-        <v>-22.2</v>
+        <v>-22.36</v>
       </c>
       <c r="N502" s="4" t="n">
         <v>5.27</v>
       </c>
       <c r="O502" s="4" t="n">
-        <v>-23.41</v>
+        <v>-23.57</v>
       </c>
       <c r="P502" s="4" t="n">
         <v>-1.06</v>
@@ -52300,7 +52294,7 @@
         </is>
       </c>
       <c r="Z502" s="4" t="n">
-        <v>39.59</v>
+        <v>39.53</v>
       </c>
       <c r="AA502" s="4" t="n">
         <v>0.2</v>
@@ -52309,7 +52303,7 @@
         <v>0</v>
       </c>
       <c r="AC502" s="4" t="n">
-        <v>60.41</v>
+        <v>60.47</v>
       </c>
       <c r="AD502" s="4" t="n">
         <v>0</v>
@@ -57049,7 +57043,7 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K72" t="n">
         <v>8</v>

</xml_diff>

<commit_message>
Add Tavern Research OH-07 poll (Aug 4-5) and rerun 2026-08-10 forecast
Tavern Research toplines (635 LV online, Aug 4-5, MoE +/-4.8) put OH-07 at
Poindexter 54 / Miller 46 on the leaner-pushed named ballot. New pollster:
an explicitly Democratic shop with no public track record, so rated 1.3
with a D house lean.

OH-07 moves R+2.41 -> R+2.3 (Dem win 40.7% -> 41.1%); nowcast has it D+2.0.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="n">
-        <v>48.4</v>
+        <v>48.7</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>233</v>
+        <v>232.8</v>
       </c>
       <c r="C9" t="n">
-        <v>202</v>
+        <v>202.2</v>
       </c>
       <c r="D9" t="n">
         <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>81.90000000000001</v>
+        <v>81.7</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.84</v>
+        <v>-3.03</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>38.1</v>
+        <v>41.9</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>61.9</v>
+        <v>58.1</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Lean R</t>
+          <t>Toss-up</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4705,13 +4705,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-2.53</v>
+        <v>-2.29</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>28.3</v>
+        <v>29.3</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>71.7</v>
+        <v>70.7</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4719,13 +4719,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.8</v>
+        <v>-2.5</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-1.3</v>
+        <v>-1</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.06</v>
@@ -4760,16 +4760,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.74</v>
+        <v>48.86</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>28.3</v>
+        <v>29.3</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.26</v>
+        <v>51.14</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -21487,7 +21487,7 @@
         </is>
       </c>
       <c r="M202" s="4" t="n">
-        <v>-17.12</v>
+        <v>-17.13</v>
       </c>
       <c r="N202" s="4" t="n">
         <v>5.29</v>
@@ -24715,7 +24715,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.05</v>
+        <v>30.23</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24729,13 +24729,13 @@
         </is>
       </c>
       <c r="M234" s="4" t="n">
-        <v>22.14</v>
+        <v>22.05</v>
       </c>
       <c r="N234" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O234" s="4" t="n">
-        <v>31.26</v>
+        <v>31.17</v>
       </c>
       <c r="P234" s="4" t="n">
         <v>1</v>
@@ -24766,10 +24766,10 @@
         <v>0</v>
       </c>
       <c r="AB234" s="4" t="n">
-        <v>62.35</v>
+        <v>62.3</v>
       </c>
       <c r="AC234" s="4" t="n">
-        <v>32.65</v>
+        <v>32.7</v>
       </c>
       <c r="AD234" s="4" t="n">
         <v>5</v>
@@ -24813,13 +24813,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.22</v>
+        <v>-3.99</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -24827,13 +24827,13 @@
         </is>
       </c>
       <c r="M235" s="4" t="n">
-        <v>-9.01</v>
+        <v>-9.1</v>
       </c>
       <c r="N235" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O235" s="4" t="n">
-        <v>-5.2</v>
+        <v>-5.28</v>
       </c>
       <c r="P235" s="4" t="n">
         <v>-0.48</v>
@@ -24870,10 +24870,10 @@
         <v>0</v>
       </c>
       <c r="AB235" s="4" t="n">
-        <v>45.42</v>
+        <v>45.39</v>
       </c>
       <c r="AC235" s="4" t="n">
-        <v>49.58</v>
+        <v>49.61</v>
       </c>
       <c r="AD235" s="4" t="n">
         <v>5</v>
@@ -28303,13 +28303,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-6.78</v>
+        <v>-6.87</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>86.8</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28317,13 +28317,13 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-12.17</v>
+        <v>-12.29</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O269" s="4" t="n">
-        <v>-8.01</v>
+        <v>-8.130000000000001</v>
       </c>
       <c r="P269" s="4" t="n">
         <v>-0.14</v>
@@ -28360,10 +28360,10 @@
         <v>0</v>
       </c>
       <c r="AB269" s="4" t="n">
-        <v>46.61</v>
+        <v>46.57</v>
       </c>
       <c r="AC269" s="4" t="n">
-        <v>53.39</v>
+        <v>53.43</v>
       </c>
       <c r="AD269" s="4" t="n">
         <v>0</v>
@@ -28411,7 +28411,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-33.74</v>
+        <v>-33.86</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28425,13 +28425,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-31.13</v>
+        <v>-31.25</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-33.74</v>
+        <v>-33.86</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28462,10 +28462,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>33.13</v>
+        <v>33.07</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>66.87</v>
+        <v>66.93000000000001</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -30057,13 +30057,13 @@
         </is>
       </c>
       <c r="I286" s="4" t="n">
-        <v>-9.140000000000001</v>
+        <v>-9.27</v>
       </c>
       <c r="J286" s="4" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="K286" s="4" t="n">
-        <v>93.7</v>
+        <v>94</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -30071,13 +30071,13 @@
         </is>
       </c>
       <c r="M286" s="4" t="n">
-        <v>-8.34</v>
+        <v>-8.5</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O286" s="4" t="n">
-        <v>-9.550000000000001</v>
+        <v>-9.710000000000001</v>
       </c>
       <c r="P286" s="4" t="n">
         <v>-0.99</v>
@@ -30114,10 +30114,10 @@
         <v>0</v>
       </c>
       <c r="AB286" s="4" t="n">
-        <v>45.43</v>
+        <v>45.36</v>
       </c>
       <c r="AC286" s="4" t="n">
-        <v>54.57</v>
+        <v>54.64</v>
       </c>
       <c r="AD286" s="4" t="n">
         <v>0</v>
@@ -30161,13 +30161,13 @@
         </is>
       </c>
       <c r="I287" s="4" t="n">
-        <v>13.09</v>
+        <v>12.96</v>
       </c>
       <c r="J287" s="4" t="n">
-        <v>99.09999999999999</v>
+        <v>99</v>
       </c>
       <c r="K287" s="4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -30175,13 +30175,13 @@
         </is>
       </c>
       <c r="M287" s="4" t="n">
-        <v>9.51</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O287" s="4" t="n">
-        <v>14.87</v>
+        <v>14.72</v>
       </c>
       <c r="P287" s="4" t="n">
         <v>0.43</v>
@@ -30218,10 +30218,10 @@
         <v>0</v>
       </c>
       <c r="AB287" s="4" t="n">
-        <v>56.55</v>
+        <v>56.48</v>
       </c>
       <c r="AC287" s="4" t="n">
-        <v>43.45</v>
+        <v>43.52</v>
       </c>
       <c r="AD287" s="4" t="n">
         <v>0</v>
@@ -30269,7 +30269,7 @@
         </is>
       </c>
       <c r="I288" s="4" t="n">
-        <v>-52.09</v>
+        <v>-52.25</v>
       </c>
       <c r="J288" s="4" t="n">
         <v>0</v>
@@ -30283,13 +30283,13 @@
         </is>
       </c>
       <c r="M288" s="4" t="n">
-        <v>-49.3</v>
+        <v>-49.45</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O288" s="4" t="n">
-        <v>-52.09</v>
+        <v>-52.25</v>
       </c>
       <c r="P288" s="4" t="n">
         <v>-2.18</v>
@@ -30320,10 +30320,10 @@
         <v>0</v>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>23.95</v>
+        <v>23.87</v>
       </c>
       <c r="AC288" s="4" t="n">
-        <v>76.05</v>
+        <v>76.13</v>
       </c>
       <c r="AD288" s="4" t="n">
         <v>0</v>
@@ -35805,13 +35805,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>1.76</v>
+        <v>2</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>68.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>31.3</v>
+        <v>30.4</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35837,16 +35837,16 @@
         <v>-11.15</v>
       </c>
       <c r="S342" s="4" t="n">
-        <v>44.77</v>
+        <v>48.25</v>
       </c>
       <c r="T342" s="4" t="n">
-        <v>38.42</v>
+        <v>41.28</v>
       </c>
       <c r="U342" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V342" s="4" t="n">
-        <v>7.44</v>
+        <v>6.52</v>
       </c>
       <c r="W342" s="5" t="n">
         <v>603156</v>
@@ -35862,10 +35862,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>50.88</v>
+        <v>51</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>49.12</v>
+        <v>49</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -47443,7 +47443,7 @@
         </is>
       </c>
       <c r="I456" s="4" t="n">
-        <v>-23.33</v>
+        <v>-23.89</v>
       </c>
       <c r="J456" s="4" t="n">
         <v>0.1</v>
@@ -47484,7 +47484,7 @@
         <v>1</v>
       </c>
       <c r="V456" s="4" t="n">
-        <v>-6</v>
+        <v>-9</v>
       </c>
       <c r="W456" s="5" t="n">
         <v>396217</v>
@@ -47500,10 +47500,10 @@
         <v>0</v>
       </c>
       <c r="AB456" s="4" t="n">
-        <v>38.33</v>
+        <v>38.06</v>
       </c>
       <c r="AC456" s="4" t="n">
-        <v>61.67</v>
+        <v>61.94</v>
       </c>
       <c r="AD456" s="4" t="n">
         <v>0</v>
@@ -48583,7 +48583,7 @@
         </is>
       </c>
       <c r="I467" s="4" t="n">
-        <v>-18.64</v>
+        <v>-19.21</v>
       </c>
       <c r="J467" s="4" t="n">
         <v>0.3</v>
@@ -48624,7 +48624,7 @@
         <v>1</v>
       </c>
       <c r="V467" s="4" t="n">
-        <v>-22</v>
+        <v>-25</v>
       </c>
       <c r="W467" s="5" t="n">
         <v>44015</v>
@@ -48640,10 +48640,10 @@
         <v>0</v>
       </c>
       <c r="AB467" s="4" t="n">
-        <v>40.68</v>
+        <v>40.39</v>
       </c>
       <c r="AC467" s="4" t="n">
-        <v>59.32</v>
+        <v>59.61</v>
       </c>
       <c r="AD467" s="4" t="n">
         <v>0</v>
@@ -49193,13 +49193,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-1.41</v>
+        <v>-0.7</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>45.5</v>
+        <v>48.4</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>54.5</v>
+        <v>51.6</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49207,13 +49207,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.78</v>
+        <v>-10.58</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.29</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-2.01</v>
+        <v>-1.8</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.43</v>
@@ -49250,10 +49250,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.4</v>
+        <v>45.45</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.6</v>
+        <v>46.55</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -50247,13 +50247,13 @@
         </is>
       </c>
       <c r="I483" s="4" t="n">
-        <v>-10.33</v>
+        <v>-10.34</v>
       </c>
       <c r="J483" s="4" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="K483" s="4" t="n">
-        <v>96.59999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="L483" t="inlineStr">
         <is>
@@ -50279,16 +50279,16 @@
         <v>-16.41</v>
       </c>
       <c r="S483" s="4" t="n">
-        <v>43.26</v>
+        <v>43.1</v>
       </c>
       <c r="T483" s="4" t="n">
-        <v>47.6</v>
+        <v>47.22</v>
       </c>
       <c r="U483" t="n">
         <v>2</v>
       </c>
       <c r="V483" s="4" t="n">
-        <v>-7.09</v>
+        <v>-7.13</v>
       </c>
       <c r="W483" s="5" t="n">
         <v>4169078</v>
@@ -50665,13 +50665,13 @@
         </is>
       </c>
       <c r="I487" s="4" t="n">
-        <v>1.62</v>
+        <v>1.19</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>68.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>31.8</v>
+        <v>33.6</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -50697,7 +50697,7 @@
         <v>7.09</v>
       </c>
       <c r="S487" s="4" t="n">
-        <v>49.75</v>
+        <v>49.19</v>
       </c>
       <c r="T487" s="4" t="n">
         <v>44.91</v>
@@ -50706,7 +50706,7 @@
         <v>6</v>
       </c>
       <c r="V487" s="4" t="n">
-        <v>3.7</v>
+        <v>2.86</v>
       </c>
       <c r="W487" s="5" t="n">
         <v>0</v>
@@ -50722,10 +50722,10 @@
         <v>0</v>
       </c>
       <c r="AB487" s="4" t="n">
-        <v>50.81</v>
+        <v>50.6</v>
       </c>
       <c r="AC487" s="4" t="n">
-        <v>49.19</v>
+        <v>49.4</v>
       </c>
       <c r="AD487" s="4" t="n">
         <v>0</v>
@@ -51089,13 +51089,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-25.42</v>
+        <v>-25.9</v>
       </c>
       <c r="J491" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51121,16 +51121,16 @@
         <v>-20.58</v>
       </c>
       <c r="S491" s="4" t="n">
-        <v>31.11</v>
+        <v>30.8</v>
       </c>
       <c r="T491" s="4" t="n">
-        <v>43.81</v>
+        <v>43.51</v>
       </c>
       <c r="U491" t="n">
         <v>6</v>
       </c>
       <c r="V491" s="4" t="n">
-        <v>-12.97</v>
+        <v>-13.03</v>
       </c>
       <c r="W491" s="5" t="n">
         <v>58829</v>
@@ -51144,16 +51144,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>14.1</v>
+        <v>14.4</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>28.41</v>
+        <v>28.02</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>53.83</v>
+        <v>53.92</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>
@@ -51305,13 +51305,13 @@
         </is>
       </c>
       <c r="I493" s="4" t="n">
-        <v>-3.66</v>
+        <v>-4.45</v>
       </c>
       <c r="J493" s="4" t="n">
-        <v>24</v>
+        <v>21.1</v>
       </c>
       <c r="K493" s="4" t="n">
-        <v>76</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="L493" t="inlineStr">
         <is>
@@ -51340,13 +51340,13 @@
         <v>47</v>
       </c>
       <c r="T493" s="4" t="n">
-        <v>42.31</v>
+        <v>42.8</v>
       </c>
       <c r="U493" t="n">
         <v>3</v>
       </c>
       <c r="V493" s="4" t="n">
-        <v>4.54</v>
+        <v>1.2</v>
       </c>
       <c r="W493" s="5" t="n">
         <v>0</v>
@@ -51360,16 +51360,16 @@
         </is>
       </c>
       <c r="Z493" s="4" t="n">
-        <v>48.17</v>
+        <v>47.78</v>
       </c>
       <c r="AA493" s="4" t="n">
-        <v>24</v>
+        <v>21.1</v>
       </c>
       <c r="AB493" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC493" s="4" t="n">
-        <v>51.83</v>
+        <v>52.22</v>
       </c>
       <c r="AD493" s="4" t="n">
         <v>0</v>
@@ -52991,7 +52991,7 @@
         <v>21</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -55135,7 +55135,7 @@
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>85</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="K39" t="n">
         <v>84</v>
@@ -55147,7 +55147,7 @@
         <v>112</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>72.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -55599,7 +55599,7 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>40.8</v>
+        <v>40.7</v>
       </c>
       <c r="K47" t="n">
         <v>41</v>
@@ -55611,7 +55611,7 @@
         <v>53</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Drop duplicate Tavern Research OH-07 poll; rerun 2026-08-15
The NYT feed picked up the Tavern Research OH-07 survey with end_date
2026-08-04, while the hand-entered copy in manual_race_polls.csv used
2026-08-05 (the PDF's own field dates are Aug 4-5). The merge dedupes on
race + pollster + end date, so the one-day gap let both survive and the
poll was counted twice.

Removed the manual row, so the feed's version is the only one and a future
scrape_race_polls won't reintroduce it. OH-07 drops from 6 polls to 5:
polling average D+1.18 -> D+0.67, margin R+3.27 -> R+3.49, dem_prob
37.5% -> 36.7%. Other race deltas are chamber-sim Monte Carlo noise.
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>51</v>
       </c>
       <c r="E8" t="n">
-        <v>56.8</v>
+        <v>56.2</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -575,7 +575,7 @@
         <v>229</v>
       </c>
       <c r="E9" t="n">
-        <v>81.2</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -591,16 +591,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.5</v>
+        <v>24.4</v>
       </c>
       <c r="C10" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="D10" t="n">
         <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>40.4</v>
+        <v>39.3</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -919,17 +919,17 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>-3.1</v>
+        <v>-3.76</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>41</v>
+        <v>38.6</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>59</v>
+        <v>61.4</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Toss-up</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M2" s="4" t="n">
@@ -4711,13 +4711,13 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>-3.18</v>
+        <v>-3.34</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>25.8</v>
+        <v>25.2</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>74.2</v>
+        <v>74.8</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4725,13 +4725,13 @@
         </is>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-2.43</v>
+        <v>-2.7</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5.32</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>-0.88</v>
+        <v>-1.14</v>
       </c>
       <c r="P38" s="4" t="n">
         <v>-1.04</v>
@@ -4766,16 +4766,16 @@
         </is>
       </c>
       <c r="Z38" s="4" t="n">
-        <v>48.41</v>
+        <v>48.33</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>25.8</v>
+        <v>25.2</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
-        <v>51.59</v>
+        <v>51.67</v>
       </c>
       <c r="AD38" s="4" t="n">
         <v>0</v>
@@ -24717,7 +24717,7 @@
         </is>
       </c>
       <c r="I234" s="4" t="n">
-        <v>30.36</v>
+        <v>30.38</v>
       </c>
       <c r="J234" s="4" t="n">
         <v>100</v>
@@ -24815,13 +24815,13 @@
         </is>
       </c>
       <c r="I235" s="4" t="n">
-        <v>-4.36</v>
+        <v>-3.99</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>35.7</v>
+        <v>38.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>64.3</v>
+        <v>61.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -28305,13 +28305,13 @@
         </is>
       </c>
       <c r="I269" s="4" t="n">
-        <v>-7.21</v>
+        <v>-7.2</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>88.2</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -28319,7 +28319,7 @@
         </is>
       </c>
       <c r="M269" s="4" t="n">
-        <v>-12.71</v>
+        <v>-12.7</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>5.32</v>
@@ -28413,7 +28413,7 @@
         </is>
       </c>
       <c r="I270" s="4" t="n">
-        <v>-34.25</v>
+        <v>-34.24</v>
       </c>
       <c r="J270" s="4" t="n">
         <v>0</v>
@@ -28427,13 +28427,13 @@
         </is>
       </c>
       <c r="M270" s="4" t="n">
-        <v>-31.67</v>
+        <v>-31.66</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>5.32</v>
       </c>
       <c r="O270" s="4" t="n">
-        <v>-34.25</v>
+        <v>-34.24</v>
       </c>
       <c r="P270" s="4" t="n">
         <v>-2.59</v>
@@ -28464,10 +28464,10 @@
         <v>0</v>
       </c>
       <c r="AB270" s="4" t="n">
-        <v>32.87</v>
+        <v>32.88</v>
       </c>
       <c r="AC270" s="4" t="n">
-        <v>67.13</v>
+        <v>67.12</v>
       </c>
       <c r="AD270" s="4" t="n">
         <v>0</v>
@@ -35807,13 +35807,13 @@
         </is>
       </c>
       <c r="I342" s="4" t="n">
-        <v>-0.7</v>
+        <v>-1.17</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>35.5</v>
+        <v>33.6</v>
       </c>
       <c r="K342" s="4" t="n">
-        <v>64.5</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -35839,16 +35839,16 @@
         <v>-11.15</v>
       </c>
       <c r="S342" s="4" t="n">
-        <v>46.08</v>
+        <v>45.02</v>
       </c>
       <c r="T342" s="4" t="n">
-        <v>42.69</v>
+        <v>42.25</v>
       </c>
       <c r="U342" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V342" s="4" t="n">
-        <v>1.18</v>
+        <v>0.67</v>
       </c>
       <c r="W342" s="5" t="n">
         <v>603156</v>
@@ -35864,10 +35864,10 @@
         <v>0</v>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>49.65</v>
+        <v>49.41</v>
       </c>
       <c r="AC342" s="4" t="n">
-        <v>50.35</v>
+        <v>50.59</v>
       </c>
       <c r="AD342" s="4" t="n">
         <v>0</v>
@@ -49195,13 +49195,13 @@
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>-0.31</v>
+        <v>-0.97</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>49.5</v>
+        <v>47.2</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>50.5</v>
+        <v>52.8</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -49209,13 +49209,13 @@
         </is>
       </c>
       <c r="M473" s="4" t="n">
-        <v>-10.6</v>
+        <v>-10.76</v>
       </c>
       <c r="N473" s="4" t="n">
         <v>5.32</v>
       </c>
       <c r="O473" s="4" t="n">
-        <v>-1.82</v>
+        <v>-1.99</v>
       </c>
       <c r="P473" s="4" t="n">
         <v>0.4</v>
@@ -49252,10 +49252,10 @@
         <v>0</v>
       </c>
       <c r="AB473" s="4" t="n">
-        <v>45.6</v>
+        <v>45.56</v>
       </c>
       <c r="AC473" s="4" t="n">
-        <v>46.4</v>
+        <v>46.44</v>
       </c>
       <c r="AD473" s="4" t="n">
         <v>8</v>
@@ -51091,7 +51091,7 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-27.57</v>
+        <v>-27.54</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
@@ -51146,13 +51146,13 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>14.27</v>
+        <v>14.24</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>27.25</v>
+        <v>27.28</v>
       </c>
       <c r="AC491" s="4" t="n">
         <v>54.82</v>
@@ -53044,7 +53044,7 @@
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="K3" t="n">
         <v>9</v>

</xml_diff>

<commit_message>
data: refresh 2026-09-04 with late-breaking FL-09 + FL-16 polls
Two SEA Polling internals landed in the NYT house feed after this
morning's scrape. Both are D-sponsored, so the average de-biases them.

FL-09 Soto 41 - Green 41 (de-biased R+3.0): D+0.25 -> R+0.68, Toss-up
FL-16 Kirschner 40 - Gruters 39 (de-biased R+2.0): R+5.13 -> R+4.16, Lean R

House D 237.7 (70.8%) - Senate D 50.4 (49.1%) - Gov D 25.5 (56.2%)

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0166PDfFpVfDzteyax1T6AK3
</commit_message>
<xml_diff>
--- a/output/nowcast.xlsx
+++ b/output/nowcast.xlsx
@@ -550,7 +550,7 @@
         <v>51</v>
       </c>
       <c r="E8" t="n">
-        <v>54.9</v>
+        <v>55.7</v>
       </c>
       <c r="F8" t="n">
         <v>51</v>
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232.6</v>
+        <v>232.3</v>
       </c>
       <c r="C9" t="n">
-        <v>202.4</v>
+        <v>202.7</v>
       </c>
       <c r="D9" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E9" t="n">
-        <v>81.3</v>
+        <v>80.7</v>
       </c>
       <c r="F9" t="n">
         <v>218</v>
@@ -600,7 +600,7 @@
         <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>66.90000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="F10" t="n">
         <v>26</v>
@@ -4724,10 +4724,10 @@
         <v>-4.89</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>81.09999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -4779,7 +4779,7 @@
         <v>44.12</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="AB38" s="4" t="n">
         <v>3.8</v>
@@ -14433,17 +14433,17 @@
         </is>
       </c>
       <c r="I133" s="4" t="n">
-        <v>0.36</v>
+        <v>-1.47</v>
       </c>
       <c r="J133" s="4" t="n">
-        <v>63.2</v>
+        <v>32.5</v>
       </c>
       <c r="K133" s="4" t="n">
-        <v>36.8</v>
+        <v>67.5</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Lean D</t>
+          <t>Lean R</t>
         </is>
       </c>
       <c r="M133" s="4" t="n">
@@ -14464,12 +14464,18 @@
       <c r="R133" s="4" t="n">
         <v>-17.93</v>
       </c>
-      <c r="S133" s="4" t="n"/>
-      <c r="T133" s="4" t="n"/>
+      <c r="S133" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="T133" s="4" t="n">
+        <v>41</v>
+      </c>
       <c r="U133" t="n">
-        <v>0</v>
-      </c>
-      <c r="V133" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="V133" s="4" t="n">
+        <v>-3</v>
+      </c>
       <c r="W133" s="5" t="n">
         <v>2157834</v>
       </c>
@@ -14484,10 +14490,10 @@
         <v>0</v>
       </c>
       <c r="AB133" s="4" t="n">
-        <v>50.18</v>
+        <v>49.26</v>
       </c>
       <c r="AC133" s="4" t="n">
-        <v>49.82</v>
+        <v>50.74</v>
       </c>
       <c r="AD133" s="4" t="n">
         <v>0</v>
@@ -15157,13 +15163,13 @@
         </is>
       </c>
       <c r="I140" s="4" t="n">
-        <v>-5.02</v>
+        <v>-3.4</v>
       </c>
       <c r="J140" s="4" t="n">
-        <v>19.1</v>
+        <v>25</v>
       </c>
       <c r="K140" s="4" t="n">
-        <v>80.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
@@ -15188,12 +15194,18 @@
       <c r="R140" s="4" t="n">
         <v>-13.81</v>
       </c>
-      <c r="S140" s="4" t="n"/>
-      <c r="T140" s="4" t="n"/>
+      <c r="S140" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="T140" s="4" t="n">
+        <v>39</v>
+      </c>
       <c r="U140" t="n">
-        <v>0</v>
-      </c>
-      <c r="V140" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="V140" s="4" t="n">
+        <v>-2</v>
+      </c>
       <c r="W140" s="5" t="n">
         <v>296507</v>
       </c>
@@ -15208,10 +15220,10 @@
         <v>0</v>
       </c>
       <c r="AB140" s="4" t="n">
-        <v>47.49</v>
+        <v>48.3</v>
       </c>
       <c r="AC140" s="4" t="n">
-        <v>52.51</v>
+        <v>51.7</v>
       </c>
       <c r="AD140" s="4" t="n">
         <v>0</v>
@@ -24842,10 +24854,10 @@
         <v>-4.59</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>20.4</v>
+        <v>20.8</v>
       </c>
       <c r="K235" s="4" t="n">
-        <v>79.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -49272,10 +49284,10 @@
         <v>-0.54</v>
       </c>
       <c r="J473" s="4" t="n">
-        <v>36.8</v>
+        <v>36.5</v>
       </c>
       <c r="K473" s="4" t="n">
-        <v>63.2</v>
+        <v>63.5</v>
       </c>
       <c r="L473" t="inlineStr">
         <is>
@@ -50744,10 +50756,10 @@
         <v>1.1</v>
       </c>
       <c r="J487" s="4" t="n">
-        <v>66.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K487" s="4" t="n">
-        <v>33.5</v>
+        <v>33.9</v>
       </c>
       <c r="L487" t="inlineStr">
         <is>
@@ -51165,13 +51177,13 @@
         </is>
       </c>
       <c r="I491" s="4" t="n">
-        <v>-27.84</v>
+        <v>-27.91</v>
       </c>
       <c r="J491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K491" s="4" t="n">
-        <v>100</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L491" t="inlineStr">
         <is>
@@ -51220,16 +51232,16 @@
         </is>
       </c>
       <c r="Z491" s="4" t="n">
-        <v>22.27</v>
+        <v>22.29</v>
       </c>
       <c r="AA491" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB491" s="4" t="n">
-        <v>23.12</v>
+        <v>23.07</v>
       </c>
       <c r="AC491" s="4" t="n">
-        <v>50.96</v>
+        <v>50.98</v>
       </c>
       <c r="AD491" s="4" t="n">
         <v>3.66</v>

</xml_diff>